<commit_message>
Audiências: sync 2026-09-23 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24E8972E-1A08-4D20-8D86-42CA994911D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{120DBA39-A601-40C7-A58A-FE3076E307C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A899EBA7-3EE3-4652-A6F1-216D7279BFBD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6D6B21FF-2EAF-46D9-8784-D252B7A6E2FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_Hlk139463631" localSheetId="0">Planilha1!$A$3</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="201">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,37 +98,298 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1000794-70.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Gabriel Goncalves Alvares</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$          2.322.472,80</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0000463-74.2026.5.14.0111</t>
+  </si>
+  <si>
+    <t>Syngenta Digital Ltda.</t>
+  </si>
+  <si>
+    <t>Lucas Rafael Chiquito De Souza</t>
+  </si>
+  <si>
+    <t>PIMENTA BUENO</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$             235.287,92</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>https://trt14-jus-br.zoom.us/j/87479999418?pwd=Dvi882AxlC4NHugWXyiLgR5Tm3zg5W.1 ID da reunião: 874 7999 9418 Senha: 986377</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1001214-26.2026.5.02.0031</t>
+  </si>
+  <si>
+    <t>Spic Brasil Energia Participações S.A.</t>
+  </si>
+  <si>
+    <t>Martha Ferreira Machado</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>31ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               40.763,68</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
+  </si>
+  <si>
+    <t>0000184-21.2025.5.05.0161</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Walney De Oliveira Rodrigues</t>
+  </si>
+  <si>
+    <t>SANTO AMARO</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>03ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$             331.871,09</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>link pendente</t>
+  </si>
+  <si>
+    <t>0000717-33.2026.5.05.0132</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Silvan Dos Anjos Dos Santos</t>
+  </si>
+  <si>
+    <t>CAMAÇARI</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$               15.684,57</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/my/sl2vtcam</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>1000970-83.2026.5.02.0068</t>
+  </si>
+  <si>
+    <t>Whirlpool S.A</t>
+  </si>
+  <si>
+    <t>Eduardo Akira Kawabata E Electrolux Do Brasil S/A</t>
+  </si>
+  <si>
+    <t>68ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               65.000,00</t>
+  </si>
+  <si>
+    <t>Grupo A3</t>
+  </si>
+  <si>
+    <t>PBS</t>
+  </si>
+  <si>
+    <t>SOF</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/81486768468?pwd=TvPkyvfbko93aYtBiWMTAIPOUojzNS.1</t>
+  </si>
+  <si>
+    <t>Audiência Una- Telepresencial</t>
+  </si>
+  <si>
+    <t>0024175-55.2026.5.24.0066</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Dionaty Sousa Dos Santos</t>
+  </si>
+  <si>
+    <t>PONTA PORÃ</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>R$               55.756,42</t>
+  </si>
+  <si>
+    <t>LWP</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/88062331360</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Presencial</t>
   </si>
   <si>
-    <t>1001200-66.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Anderson Fernando Da Silva</t>
+    <t>1001646-97.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Flavio Eduardo Basilio</t>
+  </si>
+  <si>
+    <t>R$             287.397,44</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010763-85.2025.5.03.0160</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A. - Iguatama - Igt</t>
+  </si>
+  <si>
+    <t>Marcus Vinicios Dos Santos Correia Alves</t>
+  </si>
+  <si>
+    <t>FORMIGA</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>R$               66.235,85</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>BBO</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt2formiga</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1000646-34.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Cbc - Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Danilo Domingos Da Silva</t>
   </si>
   <si>
     <t>RIBEIRÃO PIRES</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$               83.648,82</t>
+    <t>R$             121.724,54</t>
   </si>
   <si>
     <t>Grupo B3</t>
@@ -134,502 +398,253 @@
     <t>LMI</t>
   </si>
   <si>
-    <t>Presencial</t>
+    <t>0024052-57.2026.5.24.0066</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Anadirson Alem Dos Santos De Oliveira</t>
+  </si>
+  <si>
+    <t>R$             141.500,00</t>
+  </si>
+  <si>
+    <t>BTF</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/85366509499</t>
+  </si>
+  <si>
+    <t>1001307-41.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Paulo Souza De Almeida</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               80.000,00</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>1001691-98.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Daiane Silva Nascimento Dos Santos</t>
+  </si>
+  <si>
+    <t>R$             144.115,98</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>1001738-84.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda</t>
+  </si>
+  <si>
+    <t>Gregory Leonardo Fernandes</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               65.480,35</t>
+  </si>
+  <si>
+    <t>1001157-66.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Gustavo Pereira Dos Reis</t>
+  </si>
+  <si>
+    <t>R$               35.699,15</t>
   </si>
   <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>0010496-56.2026.5.15.0092</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Daniel Ferreira Souto</t>
-  </si>
-  <si>
-    <t>CAMPINAS</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          1.957.403,00</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
+    <t>0000723-50.2026.5.22.0105</t>
+  </si>
+  <si>
+    <t>Pedro Afonso Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Antonio Da Silva Sousa</t>
+  </si>
+  <si>
+    <t>PIRIPIRI</t>
+  </si>
+  <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>R$               19.164,34</t>
+  </si>
+  <si>
+    <t>https://trt22-jus-br.zoom.us/j/86414266800</t>
+  </si>
+  <si>
+    <t>0000724-35.2026.5.22.0105</t>
+  </si>
+  <si>
+    <t>Antonio Marcos Da Silva Penha</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$               19.679,83</t>
+  </si>
+  <si>
+    <t>0000725-20.2026.5.22.0105</t>
+  </si>
+  <si>
+    <t>Antonio Carlos Do Nascimento Leite</t>
+  </si>
+  <si>
+    <t>R$               17.931,44</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0000928-73.2024.5.05.0121</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A. - Candeias - Can</t>
+  </si>
+  <si>
+    <t>Eric Fabricio Dos Santos Pereira</t>
+  </si>
+  <si>
+    <t>CANDEIAS</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>R$               23.207,48</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/my/cejusc1sala18</t>
+  </si>
+  <si>
+    <t>0000447-03.2026.5.09.0195</t>
+  </si>
+  <si>
+    <t>Anderson Felipe Ferri</t>
+  </si>
+  <si>
+    <t>CASCAVEL</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             881.000,00</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/s8jj9 ID da Reunião: 83482068288 Senha: sM3uxxhDB0</t>
+  </si>
+  <si>
+    <t>Audiência de Encerramento de Instrução</t>
+  </si>
+  <si>
+    <t>0000049-63.2026.5.09.0128</t>
+  </si>
+  <si>
+    <t>Edison Luiz Souza</t>
+  </si>
+  <si>
+    <t>R$               61.000,00</t>
   </si>
   <si>
     <t>TFR</t>
   </si>
   <si>
-    <t>https://trt15-jus-br.zoom.us/j/84146096644?pwd=STloZzBJSTFaMW5PeXZRYlIrRGlIdz0</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000629-33.2026.5.02.0464</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Dario Pereira</t>
-  </si>
-  <si>
-    <t>SÃO BERNARDO DO CAMPO</t>
-  </si>
-  <si>
-    <t>04ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             310.000,00</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>VRO</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001092-71.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Edson Da Silva Morgado</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          2.126.834,60</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>0011184-68.2026.5.15.0140</t>
-  </si>
-  <si>
-    <t>Grammer Do Brasil</t>
-  </si>
-  <si>
-    <t>David Estevao Junior</t>
-  </si>
-  <si>
-    <t>ATIBAIA</t>
-  </si>
-  <si>
-    <t>R$               56.846,94</t>
+    <t>https://url.trt9.jus.br/rypyv ID da reunião: 87526086719 Senha de acesso: C9wehw1Pg0</t>
+  </si>
+  <si>
+    <t>0000183-90.2026.5.09.0128</t>
+  </si>
+  <si>
+    <t>R$             205.600,00</t>
+  </si>
+  <si>
+    <t>0010657-94.2026.5.03.0029</t>
+  </si>
+  <si>
+    <t>Sistenge Construções E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Rodrigo Junio De Souza</t>
+  </si>
+  <si>
+    <t>CONTAGEM</t>
+  </si>
+  <si>
+    <t>Acordo</t>
+  </si>
+  <si>
+    <t>R$               34.332,73</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt1.contagem</t>
+  </si>
+  <si>
+    <t>0010622-38.2026.5.15.0050</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Jeferson De Souza Alves Antonio</t>
+  </si>
+  <si>
+    <t>DRACENA</t>
+  </si>
+  <si>
+    <t>R$             323.874,68</t>
   </si>
   <si>
     <t>AAP</t>
   </si>
   <si>
-    <t>JPL</t>
-  </si>
-  <si>
-    <t>0011283-47.2025.5.15.0019</t>
-  </si>
-  <si>
-    <t>Viterra Bioenergia S.A.</t>
-  </si>
-  <si>
-    <t>Bruno Cesar Alves</t>
-  </si>
-  <si>
-    <t>ARAÇATUBA</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             319.333,36</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>Correspondente - Carla</t>
-  </si>
-  <si>
-    <t>1001101-96.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Sidnei Da Silva Dantas</t>
-  </si>
-  <si>
-    <t>R$               46.770,44</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010412-48.2026.5.03.0073</t>
-  </si>
-  <si>
-    <t>Hrz Energia</t>
-  </si>
-  <si>
-    <t>Alexandre Nery Ferreira</t>
-  </si>
-  <si>
-    <t>POÇOS DE CALDAS</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>R$             644.064,82</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
-  </si>
-  <si>
-    <t>NRG</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vt2.passos</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010265-04.2026.5.03.0176</t>
-  </si>
-  <si>
-    <t>Uhe São Simão Energia S.A.</t>
-  </si>
-  <si>
-    <t>Luis Felipe Pereira Andrade</t>
-  </si>
-  <si>
-    <t>ITUIUTABA</t>
-  </si>
-  <si>
-    <t>R$               63.000,00</t>
-  </si>
-  <si>
-    <t>ECO</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/j/83446217509</t>
-  </si>
-  <si>
-    <t>1001135-11.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Marcos Aurelio Rodrigues Goncalves</t>
-  </si>
-  <si>
-    <t>R$             807.744,00</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>0010827-38.2025.5.15.0071</t>
-  </si>
-  <si>
-    <t>Rafael Querubim Medici Amorim</t>
-  </si>
-  <si>
-    <t>MOGI GUAÇU</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>R$             331.734,05</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/5326391733?pwd=Qjc4RFBXWjZNbVd1bG5wNldjR3dWZz09</t>
-  </si>
-  <si>
-    <t>1000533-30.2026.5.02.0363</t>
-  </si>
-  <si>
-    <t>Renato Fernandes Heleno</t>
-  </si>
-  <si>
-    <t>MAUÁ</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             571.654,41</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>0010620-68.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>Marcio Aragao De Melo</t>
-  </si>
-  <si>
-    <t>DRACENA</t>
-  </si>
-  <si>
-    <t>R$               35.458,88</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
     <t>https://trt15-jus.br.zoom.us/j/87527564652?pwd=d3YrZ2diWXk5UjgzbmVkNExteWVMQT09</t>
   </si>
   <si>
-    <t>0010089-36.2026.5.15.0129</t>
-  </si>
-  <si>
-    <t>Lucas De Oliveira Lima</t>
-  </si>
-  <si>
-    <t>10ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$               32.965,01</t>
-  </si>
-  <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>Presencial | Advogada - Dra. Isis Zuri, (19) 99287-5454 | Preposta - Juliana da Silva Oliveira, CPF 285.253.868-71, RG 359894124, (19) 98743-4081</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010625-64.2021.5.15.0083</t>
-  </si>
-  <si>
-    <t>Yaborã Indústria Aeronáutica S.A.</t>
-  </si>
-  <si>
-    <t>Rogerio Nacimento Costa Pinto</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>03ª TURMA</t>
-  </si>
-  <si>
-    <t>Recursal</t>
-  </si>
-  <si>
-    <t>R$             193.321,78</t>
-  </si>
-  <si>
-    <t>BCF</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/89948955228?pwd=Vxka0xpnjrrjCMbWqVbY0TE64PtkXn.1</t>
-  </si>
-  <si>
-    <t>0010499-82.2026.5.15.0133</t>
-  </si>
-  <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Jose Luiz Dos Santos</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DO RIO PRETO</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>R$             471.779,49</t>
-  </si>
-  <si>
-    <t>GVM</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/7871570572?pwd=KzBzUnVURkZwc0gxd21YU3pUWWhJQT09</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>0012204-93.2025.5.15.0087</t>
-  </si>
-  <si>
-    <t>Renato Ranulfo Seviolla Magalhaes</t>
-  </si>
-  <si>
-    <t>PAULÍNIA</t>
-  </si>
-  <si>
-    <t>R$             372.859,54</t>
-  </si>
-  <si>
-    <t>JRM</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/85267876480?pwd=tETOC8GDaqZZdf9WNGOaW98aPE2MQx.1</t>
-  </si>
-  <si>
-    <t>0011355-05.2026.5.15.0082</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Moema</t>
-  </si>
-  <si>
-    <t>Floresvaldo Sampaio</t>
-  </si>
-  <si>
-    <t>R$             162.160,00</t>
-  </si>
-  <si>
-    <t>LWP</t>
+    <t>0010451-53.2026.5.15.0027</t>
+  </si>
+  <si>
+    <t>Guariroba Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Valdeir Cesar De Oliveira</t>
+  </si>
+  <si>
+    <t>VOTUPORANGA</t>
+  </si>
+  <si>
+    <t>R$             474.192,34</t>
   </si>
   <si>
     <t>https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1</t>
-  </si>
-  <si>
-    <t>0010628-45.2026.5.15.0050</t>
-  </si>
-  <si>
-    <t>Jose Graciel Felix De Souza</t>
-  </si>
-  <si>
-    <t>R$               64.436,81</t>
-  </si>
-  <si>
-    <t>RYL</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Presencial</t>
-  </si>
-  <si>
-    <t>0010928-75.2025.5.15.0071</t>
-  </si>
-  <si>
-    <t>Mislene Santos Do Nascimento</t>
-  </si>
-  <si>
-    <t>04ª TURMA</t>
-  </si>
-  <si>
-    <t>R$             763.302,38</t>
-  </si>
-  <si>
-    <t>KBM</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/81338233394?pwd=9sZYKqQDl9HW1PQRiyWxtnDNoRMuzq.1 ID da reunião: 813 3823 3394 Senha: 181436</t>
-  </si>
-  <si>
-    <t>0010480-82.2025.5.15.0013</t>
-  </si>
-  <si>
-    <t>Embraer S.A.</t>
-  </si>
-  <si>
-    <t>Paulo Pereira Cabral Da Silva</t>
-  </si>
-  <si>
-    <t>R$               39.651,24</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>0010408-53.2026.5.03.0156</t>
-  </si>
-  <si>
-    <t>Itapagipe Bioenergia Ltda.</t>
-  </si>
-  <si>
-    <t>Bruno Da Silva Maia</t>
-  </si>
-  <si>
-    <t>FRUTAL</t>
-  </si>
-  <si>
-    <t>R$             100.607,86</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vtfrutal</t>
-  </si>
-  <si>
-    <t>1002113-47.2024.5.02.0434</t>
-  </si>
-  <si>
-    <t>Felipe Eduardo Albano De Freitas</t>
-  </si>
-  <si>
-    <t>CEJUSC ABC</t>
-  </si>
-  <si>
-    <t>Execução</t>
-  </si>
-  <si>
-    <t>R$             660.679,72</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/86579309928?pwd=ZXdjSDg5U0llVFZYWktxT3h5SzRRZz09 ID da reunião: 865 7930 9928 Senha de acesso: 171003</t>
-  </si>
-  <si>
-    <t>0010656-76.2026.5.15.0126</t>
-  </si>
-  <si>
-    <t>Manoel Messias Ferreira</t>
-  </si>
-  <si>
-    <t>R$             242.003,29</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/83352065501?pwd=Lzc2WUJGSVpVWmJyZjB3Y0NvUmJPZz09</t>
-  </si>
-  <si>
-    <t>0011217-57.2023.5.15.0045</t>
-  </si>
-  <si>
-    <t>Valmir Henrique Franca</t>
-  </si>
-  <si>
-    <t>CEJUSC TST</t>
-  </si>
-  <si>
-    <t>Recursal TST</t>
-  </si>
-  <si>
-    <t>R$             752.419,84</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>bit.ly/Cejusc2026</t>
   </si>
 </sst>
 </file>
@@ -1094,30 +1109,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC6FEC1-4DBD-4FE8-A541-E3012D8A8A90}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4BA9B5F-64AD-40BE-A136-29A2274B0B14}">
   <dimension ref="A1:R26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="52.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="99.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="101" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,13 +1190,13 @@
     </row>
     <row r="2" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>105869</v>
+        <v>104857</v>
       </c>
       <c r="B2" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C2" s="6">
-        <v>0.3611111111111111</v>
+        <v>0.36805555555555558</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -1223,45 +1238,45 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R2" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>106141</v>
+        <v>105754</v>
       </c>
       <c r="B3" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C3" s="6">
-        <v>0.3611111111111111</v>
+        <v>0.375</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -1270,51 +1285,51 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>104807</v>
+        <v>105874</v>
       </c>
       <c r="B4" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C4" s="6">
         <v>0.375</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>25</v>
@@ -1326,54 +1341,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
-        <v>105231</v>
+        <v>103592</v>
       </c>
       <c r="B5" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.375</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1382,54 +1397,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>104933</v>
+        <v>105674</v>
       </c>
       <c r="B6" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C6" s="6">
-        <v>0.44791666666666669</v>
+        <v>0.38194444444444442</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1438,51 +1453,51 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>103325</v>
+        <v>105272</v>
       </c>
       <c r="B7" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C7" s="6">
-        <v>0.4513888888888889</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>25</v>
@@ -1494,51 +1509,51 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>31</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>105668</v>
+        <v>104492</v>
       </c>
       <c r="B8" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C8" s="6">
-        <v>0.4513888888888889</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>25</v>
@@ -1550,51 +1565,51 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>105368</v>
+        <v>105935</v>
       </c>
       <c r="B9" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C9" s="6">
-        <v>0.45833333333333331</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>25</v>
@@ -1606,51 +1621,51 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>87</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>104575</v>
+        <v>102444</v>
       </c>
       <c r="B10" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C10" s="6">
-        <v>0.46527777777777779</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>25</v>
@@ -1662,51 +1677,51 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>105261</v>
+        <v>104855</v>
       </c>
       <c r="B11" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C11" s="6">
-        <v>0.47222222222222221</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>42</v>
+        <v>110</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>53</v>
+        <v>112</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>25</v>
@@ -1718,54 +1733,54 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>101325</v>
+        <v>104198</v>
       </c>
       <c r="B12" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C12" s="6">
-        <v>0.49305555555555558</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>44</v>
+        <v>119</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>102</v>
+        <v>120</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="L12" s="7" t="s">
         <v>26</v>
@@ -1774,51 +1789,51 @@
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>104806</v>
+        <v>105579</v>
       </c>
       <c r="B13" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C13" s="6">
-        <v>0.49305555555555558</v>
+        <v>0.4375</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>25</v>
@@ -1830,45 +1845,45 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>59</v>
+        <v>130</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>104967</v>
+        <v>105955</v>
       </c>
       <c r="B14" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C14" s="6">
-        <v>0.54166666666666663</v>
+        <v>0.4513888888888889</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>116</v>
+        <v>22</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>23</v>
@@ -1886,51 +1901,51 @@
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>118</v>
+        <v>30</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>120</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>103814</v>
+        <v>106017</v>
       </c>
       <c r="B15" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C15" s="6">
-        <v>0.54861111111111116</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>53</v>
+        <v>136</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>25</v>
@@ -1942,54 +1957,54 @@
         <v>27</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>125</v>
+        <v>31</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>100</v>
+        <v>134</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>126</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>79991</v>
+        <v>105295</v>
       </c>
       <c r="B16" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C16" s="6">
-        <v>0.5625</v>
+        <v>0.46180555555555558</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>129</v>
+        <v>20</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>131</v>
+        <v>22</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>26</v>
@@ -1998,54 +2013,54 @@
         <v>27</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="R16" s="7" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
-        <v>104334</v>
+        <v>105544</v>
       </c>
       <c r="B17" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C17" s="6">
-        <v>0.58333333333333337</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>78</v>
+        <v>143</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>141</v>
+        <v>25</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>26</v>
@@ -2054,54 +2069,54 @@
         <v>27</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
-        <v>103649</v>
+        <v>105545</v>
       </c>
       <c r="B18" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C18" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.4826388888888889</v>
       </c>
       <c r="D18" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>138</v>
-      </c>
       <c r="G18" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="I18" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J18" s="7" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="L18" s="7" t="s">
         <v>26</v>
@@ -2110,54 +2125,54 @@
         <v>27</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="P18" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="R18" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="Q18" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="R18" s="7" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
-        <v>105341</v>
+        <v>105546</v>
       </c>
       <c r="B19" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C19" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F19" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K19" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="K19" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L19" s="7" t="s">
         <v>26</v>
@@ -2166,54 +2181,54 @@
         <v>27</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>156</v>
+        <v>123</v>
       </c>
       <c r="R19" s="7" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
-        <v>104968</v>
+        <v>102261</v>
       </c>
       <c r="B20" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C20" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.4861111111111111</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>78</v>
+        <v>158</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>68</v>
+        <v>160</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>116</v>
+        <v>162</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>24</v>
+        <v>163</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>26</v>
@@ -2222,54 +2237,54 @@
         <v>27</v>
       </c>
       <c r="N20" s="7" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="O20" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>161</v>
+        <v>108</v>
       </c>
       <c r="R20" s="7" t="s">
-        <v>120</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
-        <v>101050</v>
+        <v>104518</v>
       </c>
       <c r="B21" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C21" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.5625</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>162</v>
+        <v>33</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>103</v>
+        <v>168</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>23</v>
+        <v>169</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="L21" s="7" t="s">
         <v>26</v>
@@ -2278,54 +2293,54 @@
         <v>27</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="R21" s="7" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
-        <v>100167</v>
+        <v>103768</v>
       </c>
       <c r="B22" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C22" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.5625</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="E22" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J22" s="7" t="s">
-        <v>165</v>
+        <v>69</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>133</v>
+        <v>25</v>
       </c>
       <c r="L22" s="7" t="s">
         <v>26</v>
@@ -2334,51 +2349,51 @@
         <v>27</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>85</v>
+        <v>52</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
-        <v>104959</v>
+        <v>104017</v>
       </c>
       <c r="B23" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C23" s="6">
-        <v>0.61111111111111116</v>
+        <v>0.56319444444444444</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>78</v>
+        <v>173</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F23" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>176</v>
-      </c>
       <c r="H23" s="7" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>83</v>
+        <v>169</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>25</v>
@@ -2390,54 +2405,54 @@
         <v>27</v>
       </c>
       <c r="N23" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="O23" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="R23" s="7" t="s">
         <v>178</v>
-      </c>
-      <c r="O23" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="P23" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q23" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="R23" s="7" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="24" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
-        <v>99358</v>
+        <v>104768</v>
       </c>
       <c r="B24" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C24" s="6">
-        <v>0.65555555555555556</v>
+        <v>0.59375</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>88</v>
+        <v>158</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>53</v>
+        <v>182</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>55</v>
+        <v>184</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>23</v>
+        <v>105</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>182</v>
+        <v>138</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="L24" s="7" t="s">
         <v>26</v>
@@ -2446,54 +2461,54 @@
         <v>27</v>
       </c>
       <c r="N24" s="7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="O24" s="7" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="R24" s="7" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
-        <v>104930</v>
+        <v>105106</v>
       </c>
       <c r="B25" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C25" s="6">
-        <v>0.67361111111111116</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>145</v>
+        <v>33</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>138</v>
+        <v>189</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>148</v>
+        <v>191</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>141</v>
+        <v>70</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>26</v>
@@ -2502,54 +2517,54 @@
         <v>27</v>
       </c>
       <c r="N25" s="7" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="O25" s="7" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>66</v>
+        <v>193</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>143</v>
+        <v>193</v>
       </c>
       <c r="R25" s="7" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
-        <v>95035</v>
+        <v>104811</v>
       </c>
       <c r="B26" s="5">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="C26" s="6">
-        <v>0.68055555555555558</v>
+        <v>0.63541666666666663</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>88</v>
+        <v>33</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>170</v>
+        <v>196</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>131</v>
+        <v>198</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>192</v>
+        <v>39</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>193</v>
+        <v>25</v>
       </c>
       <c r="L26" s="7" t="s">
         <v>26</v>
@@ -2558,38 +2573,39 @@
         <v>27</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>195</v>
+        <v>123</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>195</v>
+        <v>74</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R3" r:id="rId1" xr:uid="{21390778-6B75-4737-BBF0-016C2BC00A37}"/>
-    <hyperlink ref="R9" r:id="rId2" xr:uid="{AAAE512A-B78E-4531-962D-BD2BE128CA20}"/>
-    <hyperlink ref="R10" r:id="rId3" xr:uid="{F795E5B6-5162-4CD5-8F9D-24AA106958F2}"/>
-    <hyperlink ref="R12" r:id="rId4" xr:uid="{31523305-119F-4B4A-83EA-ED37981E65B4}"/>
-    <hyperlink ref="R14" r:id="rId5" xr:uid="{F1833C40-B8B5-4BF0-A281-29379D2E307A}"/>
-    <hyperlink ref="R16" r:id="rId6" xr:uid="{12737FC0-59B3-4D41-B038-877F94886E44}"/>
-    <hyperlink ref="R17" r:id="rId7" xr:uid="{688E861C-3DA6-4E58-BC84-316E52BDB333}"/>
-    <hyperlink ref="R18" r:id="rId8" xr:uid="{DB3BD961-3D16-4085-85E0-CCFE7F1F6F7A}"/>
-    <hyperlink ref="R19" r:id="rId9" xr:uid="{1D600027-95A5-42D9-B3C3-7ECBEBCF1E8B}"/>
-    <hyperlink ref="R20" r:id="rId10" xr:uid="{CCDC4D54-A201-4377-8698-74741A7985E6}"/>
-    <hyperlink ref="R21" r:id="rId11" display="https://trt15-jus-br.zoom.us/j/81338233394?pwd=9sZYKqQDl9HW1PQRiyWxtnDNoRMuzq.1%20ID%20da%20reunião:%20813%203823%203394%20Senha:%20181436" xr:uid="{F1142A8A-F128-4FBD-8F21-AF02939D23F1}"/>
-    <hyperlink ref="R22" r:id="rId12" display="https://trt15-jus-br.zoom.us/j/81338233394?pwd=9sZYKqQDl9HW1PQRiyWxtnDNoRMuzq.1%20ID%20da%20reunião:%20813%203823%203394%20Senha:%20181436" xr:uid="{57711ECA-04ED-4D43-8768-7703BCA0506E}"/>
-    <hyperlink ref="R23" r:id="rId13" xr:uid="{4DE35AFD-F454-4875-A32A-C963088278B6}"/>
-    <hyperlink ref="R24" r:id="rId14" display="https://trt2-jus-br.zoom.us/j/86579309928?pwd=ZXdjSDg5U0llVFZYWktxT3h5SzRRZz09%20ID%20da%20reunião:%20865%207930%209928%20Senha%20de%20acesso:%20171003" xr:uid="{B1DA8C29-1140-4F09-AB5C-D7EBC161A31E}"/>
-    <hyperlink ref="R25" r:id="rId15" xr:uid="{5708E9C2-AEBF-413A-BF6D-9D265BBA5E59}"/>
+    <hyperlink ref="R3" r:id="rId1" display="https://trt14-jus-br.zoom.us/j/87479999418?pwd=Dvi882AxlC4NHugWXyiLgR5Tm3zg5W.1%20ID%20da%20reunião:%20874%207999%209418%20Senha:%20986377" xr:uid="{673EF94E-78A6-492F-8648-55A3D099E909}"/>
+    <hyperlink ref="R6" r:id="rId2" xr:uid="{AA314538-1C38-4354-86E5-68E87B982D8E}"/>
+    <hyperlink ref="R7" r:id="rId3" xr:uid="{2994172D-10B1-4E38-8B17-6E40060423C8}"/>
+    <hyperlink ref="R8" r:id="rId4" xr:uid="{337F0E7C-9834-4F6A-9366-2EE1C8C3ED34}"/>
+    <hyperlink ref="R10" r:id="rId5" xr:uid="{39C64E5E-477A-4E44-89F4-F4BDC7900F55}"/>
+    <hyperlink ref="R12" r:id="rId6" xr:uid="{BC5523E5-17AF-4C68-A62F-E6DF014877CF}"/>
+    <hyperlink ref="R17" r:id="rId7" display="https://trt24-jus-br.zoom.us/j/85366509499" xr:uid="{DB0C2D5F-E147-4E7A-8BE4-F33AE0556B4F}"/>
+    <hyperlink ref="R18" r:id="rId8" display="https://trt24-jus-br.zoom.us/j/85366509499" xr:uid="{491C03DC-F319-4A89-97E1-7591FFD1A851}"/>
+    <hyperlink ref="R19" r:id="rId9" display="https://trt24-jus-br.zoom.us/j/85366509499" xr:uid="{6881F188-59F0-4EF1-99F9-84F5B01E0687}"/>
+    <hyperlink ref="R20" r:id="rId10" xr:uid="{C40BC2D4-5634-4A74-BD93-2B0CB2A7D70C}"/>
+    <hyperlink ref="R21" r:id="rId11" xr:uid="{40E68771-6D02-4BFF-9A46-E2B165D419BF}"/>
+    <hyperlink ref="R22" r:id="rId12" xr:uid="{F94979A7-0CE2-472D-85F0-6E4C831FD8B8}"/>
+    <hyperlink ref="R23" r:id="rId13" xr:uid="{C4163228-EBAE-4ACB-9A5A-BF01A833E4C2}"/>
+    <hyperlink ref="R24" r:id="rId14" xr:uid="{8E3D49F9-3FE0-4C21-9505-73904F08F907}"/>
+    <hyperlink ref="R25" r:id="rId15" xr:uid="{93E3311E-435F-49CB-9DDA-D716D182C785}"/>
+    <hyperlink ref="R26" r:id="rId16" xr:uid="{0905EEA3-9A4C-4F86-82A7-9C748403172B}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-09-28 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEE00D9F-36E1-4979-B942-8AA30026107F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{49334A71-1D9C-442E-881A-F50F700FA893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8406919-E204-4FFE-A1BD-A8C2FFC627D7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{71ACA0ED-DFD1-4CCA-81B3-5204ACD80980}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="164">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,274 +95,449 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0000504-21.2026.5.18.0211</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda.</t>
+  </si>
+  <si>
+    <t>Dayanne Campera</t>
+  </si>
+  <si>
+    <t>FORMOSA</t>
+  </si>
+  <si>
+    <t>GO</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$          1.152.545,37</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>https://trt18-jus-br.zoom.us/j/86900317711</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1001393-07.2026.5.02.0080</t>
+  </si>
+  <si>
+    <t>L. Sant'Angelo Pinturas Ltda.</t>
+  </si>
+  <si>
+    <t>Tiago De Souza Vieira</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>80ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$               45.292,92</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>0011544-18.2025.5.15.0017</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Anderson Sanches Dos Santos</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>R$               60.797,04</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81715388288?pwd=UFAwUGVFQkN1bGNXcStQUEovR2VZUT09 ID da Reunião 817 1538 8288 Senha 198674</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>0011229-05.2026.5.03.0044</t>
-  </si>
-  <si>
-    <t>Syngenta Seeds Ltda.</t>
-  </si>
-  <si>
-    <t>Gilvania Ferraz</t>
-  </si>
-  <si>
-    <t>UBERLÂNDIA</t>
+    <t>0010832-56.2026.5.03.0072</t>
+  </si>
+  <si>
+    <t>Usina Fotovoltaica Arinos</t>
+  </si>
+  <si>
+    <t>Leonardo Rocha Braga</t>
+  </si>
+  <si>
+    <t>PIRAPORA</t>
   </si>
   <si>
     <t>MG</t>
   </si>
   <si>
+    <t>R$          1.018.759,39</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/j/87213692922</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0021040-47.2025.5.04.0124</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A.</t>
+  </si>
+  <si>
+    <t>Wesley Astrogildo Alves</t>
+  </si>
+  <si>
+    <t>RIO GRANDE</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               23.800,00</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
+    <t>BBO</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Luciane Veiga Cozza Neves lucianecozza@gmail.com 53984740466</t>
+  </si>
+  <si>
+    <t>0021125-33.2025.5.04.0124</t>
+  </si>
+  <si>
+    <t>R$             180.000,00</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>0012834-08.2024.5.15.0016</t>
+  </si>
+  <si>
+    <t>De Nora Do Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Luiz Henrique Marques De Arruda</t>
+  </si>
+  <si>
+    <t>SOROCABA</t>
+  </si>
+  <si>
     <t>02ª VARA DO TRABALHO</t>
   </si>
   <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             600.000,00</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
+    <t>R$               64.530,11</t>
+  </si>
+  <si>
+    <t>AAP</t>
   </si>
   <si>
     <t>JPL</t>
   </si>
   <si>
-    <t>GVM</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/j/89965522514?pwd=E84WVH0QChjzl3IpQzW7Z5L8So4lbA.1</t>
-  </si>
-  <si>
-    <t>Perícia Técnica</t>
-  </si>
-  <si>
-    <t>0012958-34.2025.5.15.0152</t>
-  </si>
-  <si>
-    <t>Dell Computadores Do Brasil Ltda.</t>
-  </si>
-  <si>
-    <t>Daisy Ferreira Da Silva</t>
-  </si>
-  <si>
-    <t>HORTOLÂNDIA</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>R$             218.600,00</t>
-  </si>
-  <si>
-    <t>AAP</t>
-  </si>
-  <si>
-    <t>Iremos acompanhar</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001633-10.2026.5.02.0431</t>
+    <t>https://trt15-jus-br.zoom.us/j/87095656771?pwd=aU9LaTBPcFd4aFAydkZSRVlpcWlRQT09 ID da reunião: 87095656771 Senha de acesso: 493462</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>0000439-62.2026.5.05.0122</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A</t>
+  </si>
+  <si>
+    <t>Vagner Bitencourt Dantas</t>
+  </si>
+  <si>
+    <t>CANDEIAS</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             115.000,00</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/j/81384816334?pwd=apkqLttWhpydFq87kabYZHeapeGXQE.1</t>
+  </si>
+  <si>
+    <t>1001194-59.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Darcio Junior De Souza Oliveira</t>
+  </si>
+  <si>
+    <t>RIBEIRÃO PIRES</t>
+  </si>
+  <si>
+    <t>R$               56.580,72</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0000112-27.2025.5.19.0005</t>
+  </si>
+  <si>
+    <t>Pedro Afonso Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Gildo Florencio De Melo</t>
+  </si>
+  <si>
+    <t>MACEIÓ</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>CEJUSC 2º GRAU</t>
+  </si>
+  <si>
+    <t>R$             123.314,66</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://trt19-jus-br.zoom.us/my/cejusc02</t>
+  </si>
+  <si>
+    <t>1000773-09.2026.5.02.0431</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>Irinaldo Jose Barbosa Da Silva</t>
+    <t>Jonathan Wanus Batista Santos</t>
   </si>
   <si>
     <t>SANTO ANDRÉ</t>
   </si>
   <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             666.224,50</t>
+    <t>R$             138.909,67</t>
   </si>
   <si>
     <t>Grupo B1</t>
   </si>
   <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>TAM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>1001298-51.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Bianca Carvalho De Macedo</t>
-  </si>
-  <si>
-    <t>RIBEIRÃO PIRES</t>
-  </si>
-  <si>
-    <t>R$             573.916,58</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>LMI</t>
-  </si>
-  <si>
-    <t>1001290-74.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Deoclecio Queiroz Batista</t>
-  </si>
-  <si>
-    <t>R$             225.333,51</t>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>Audiência Una- Telepresencial</t>
+  </si>
+  <si>
+    <t>0010626-75.2025.5.15.0126</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Joao Paulo Paiva Azevedo</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>R$             122.179,31</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09 ID da reunião: 997 370 0634 Senha: 592209</t>
+  </si>
+  <si>
+    <t>0024912-96.2026.5.24.0021</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Eduardo Galdino De Souza Junior</t>
+  </si>
+  <si>
+    <t>DOURADOS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>R$             351.071,44</t>
+  </si>
+  <si>
+    <t>BTF</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/my/trt24douvt1sala2</t>
   </si>
   <si>
     <t>Audiência Inicial - Semipresencial</t>
   </si>
   <si>
-    <t>1001006-66.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Cbc - Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Fernando Aparecido Pimenta</t>
-  </si>
-  <si>
-    <t>R$             154.012,70</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>1001258-69.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Patricia Da Silva Martins</t>
-  </si>
-  <si>
-    <t>R$               92.029,52</t>
-  </si>
-  <si>
-    <t>1001303-73.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Alexsandro Oliveira Lima</t>
-  </si>
-  <si>
-    <t>R$             148.019,33</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0016948-37.2026.5.16.0001</t>
-  </si>
-  <si>
-    <t>Fertilizantes Tocantins S.A</t>
-  </si>
-  <si>
-    <t>Jorge Rayr Goncalves Do Nascimento</t>
-  </si>
-  <si>
-    <t>SÃO LUIS</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>R$             218.153,71</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>Correspondente - doc9</t>
-  </si>
-  <si>
-    <t>RYL</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Presencial | Advogada - Raiane Costa Correia </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF467886"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>raianecorreia.adv@hotmail.com</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 98985305143 | Preposto - Katicianne da Encarnação Ferreira </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF467886"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>correspondenciasferreira30@gmail.com</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 98 70231725</t>
-    </r>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000681-91.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Bruno Henrique Rossani</t>
-  </si>
-  <si>
-    <t>R$             163.554,59</t>
+    <t>0001060-98.2026.5.17.0001</t>
+  </si>
+  <si>
+    <t>Jose Rodrigues Pereira</t>
+  </si>
+  <si>
+    <t>VITÓRIA</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>R$               76.053,43</t>
+  </si>
+  <si>
+    <t>https://trt17-jus-br.zoom.us/j/88071082197?pwd=3Jyy9TzvvP7udba72jiNuaL9ge2cbv.1</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0024341-87.2026.5.24.0066</t>
+  </si>
+  <si>
+    <t>Adriano Da Paixao Silva</t>
+  </si>
+  <si>
+    <t>PONTA PORÃ</t>
+  </si>
+  <si>
+    <t>R$               37.755,18</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/88280656823</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011020-25.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Jadir Goncalves Junior</t>
+  </si>
+  <si>
+    <t>PATROCÍNIO</t>
+  </si>
+  <si>
+    <t>R$             313.300,00</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
+  </si>
+  <si>
+    <t>0000475-80.2026.5.10.0861</t>
+  </si>
+  <si>
+    <t>Pedro Afonso Acucar &amp; Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Ronildo Raposo Bastos</t>
+  </si>
+  <si>
+    <t>GUARAÍ</t>
+  </si>
+  <si>
+    <t>TO</t>
+  </si>
+  <si>
+    <t>R$               92.000,00</t>
+  </si>
+  <si>
+    <t>Correspondente</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Claudia Rafaela Vieira claudiarafaelav@hotmail.com 63 99930-0380</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -380,12 +555,6 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF467886"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -452,16 +621,14 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFBFBFBF"/>
+        <color indexed="64"/>
       </left>
       <right style="medium">
-        <color rgb="FFBFBFBF"/>
+        <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color rgb="FFBFBFBF"/>
-      </top>
+      <top/>
       <bottom style="medium">
-        <color rgb="FFBFBFBF"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -470,9 +637,7 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -481,7 +646,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -506,7 +671,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -843,11 +1008,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7507D9D-F2E3-4822-8706-B52CC5514B69}">
-  <dimension ref="A1:R11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB99119E-E3CC-43FC-8617-A2A6D6422781}">
+  <dimension ref="A1:R18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -903,12 +1087,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>105527</v>
+        <v>104347</v>
       </c>
       <c r="B2" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C2" s="6">
         <v>0.33333333333333331</v>
@@ -953,45 +1137,45 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R2" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="R2" s="8" t="s">
+    </row>
+    <row r="3" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>105842</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.34722222222222221</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>103560</v>
-      </c>
-      <c r="B3" s="5">
-        <v>46290</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="K3" s="7" t="s">
         <v>39</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>40</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -1000,54 +1184,54 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="P3" s="7" t="s">
         <v>42</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="R3" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>105857</v>
+        <v>101961</v>
       </c>
       <c r="B4" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C4" s="6">
-        <v>0.36458333333333331</v>
+        <v>0.36805555555555558</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="7" t="s">
+      <c r="K4" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>40</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -1059,51 +1243,51 @@
         <v>50</v>
       </c>
       <c r="O4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="R4" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>106156</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.38194444444444442</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R4" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>106013</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46290</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.375</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="J5" s="7" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1112,54 +1296,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="P5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="R5" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="Q5" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="R5" s="8" t="s">
-        <v>54</v>
-      </c>
     </row>
-    <row r="6" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>105995</v>
+        <v>103302</v>
       </c>
       <c r="B6" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C6" s="6">
-        <v>0.38194444444444442</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1168,54 +1352,54 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="R6" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>103580</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.40972222222222221</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="O6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="R6" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4">
-        <v>105505</v>
-      </c>
-      <c r="B7" s="5">
-        <v>46290</v>
-      </c>
-      <c r="C7" s="6">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="I7" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="J7" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>39</v>
-      </c>
       <c r="K7" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>26</v>
@@ -1224,54 +1408,54 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>105949</v>
+        <v>99247</v>
       </c>
       <c r="B8" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C8" s="6">
-        <v>0.40277777777777779</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1280,54 +1464,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>106021</v>
+        <v>105260</v>
       </c>
       <c r="B9" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C9" s="6">
-        <v>0.40972222222222221</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1336,54 +1520,54 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>104853</v>
+        <v>105848</v>
       </c>
       <c r="B10" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C10" s="6">
         <v>0.41666666666666669</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="J10" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>40</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
@@ -1392,54 +1576,54 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="R10" s="8" t="s">
-        <v>88</v>
+        <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>104946</v>
+        <v>99928</v>
       </c>
       <c r="B11" s="5">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="C11" s="6">
-        <v>0.4236111111111111</v>
+        <v>0.42708333333333331</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>57</v>
+        <v>104</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>59</v>
+        <v>106</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>38</v>
+        <v>107</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>39</v>
+        <v>108</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>26</v>
@@ -1448,26 +1632,430 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>62</v>
+        <v>110</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="R11" s="8" t="s">
-        <v>54</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>104809</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.4861111111111111</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="R12" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>100924</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="R13" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>105019</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="R14" s="8" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>105568</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="R15" s="8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>105432</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.59375</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>105998</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.60069444444444442</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>105893</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46293</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="R18" s="8" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" xr:uid="{FEE4FA16-F4EF-4884-84C9-5E21EDF0EF3F}"/>
+    <hyperlink ref="R2" r:id="rId1" xr:uid="{95C41F58-3842-4941-84C0-4E41CF3BF528}"/>
+    <hyperlink ref="R4" r:id="rId2" display="https://trt15-jus-br.zoom.us/j/81715388288?pwd=UFAwUGVFQkN1bGNXcStQUEovR2VZUT09%20ID%20da%20Reunião%20817%201538%208288%20Senha%20198674" xr:uid="{66F6AC30-2DD9-4D73-A693-58FD44C7E513}"/>
+    <hyperlink ref="R5" r:id="rId3" xr:uid="{F28160D0-1A3B-4008-93FB-5D6BA38DCEA6}"/>
+    <hyperlink ref="R6" r:id="rId4" display="mailto:lucianecozza@gmail.com" xr:uid="{B07A87C9-1834-49BD-9549-EF7989F4D3F2}"/>
+    <hyperlink ref="R7" r:id="rId5" display="mailto:lucianecozza@gmail.com" xr:uid="{F5744966-D984-4380-86DB-E4714149FD62}"/>
+    <hyperlink ref="R8" r:id="rId6" display="https://trt15-jus-br.zoom.us/j/87095656771?pwd=aU9LaTBPcFd4aFAydkZSRVlpcWlRQT09%20ID%20da%20reunião:%2087095656771%20Senha%20de%20acesso:%20493462" xr:uid="{935FB631-F272-4CC4-B92D-6F73074C488A}"/>
+    <hyperlink ref="R9" r:id="rId7" xr:uid="{8D9DD257-B0B0-43F8-83EE-C8694A826464}"/>
+    <hyperlink ref="R11" r:id="rId8" xr:uid="{C865ADBB-9361-4C89-A64E-9BF22550947D}"/>
+    <hyperlink ref="R13" r:id="rId9" display="https://trt15-jus-br.zoom.us/j/9973700634?pwd=dENDekhCNjFLekRnSExiTzhmK1VLdz09%20ID%20da%20reunião:%20997%20370%200634%20Senha:%20592209" xr:uid="{6CF8C3D3-A3B6-4309-9DBC-94DB4B1068ED}"/>
+    <hyperlink ref="R14" r:id="rId10" xr:uid="{5FB6E6AA-19E1-4D53-A5B8-AE44970377D1}"/>
+    <hyperlink ref="R15" r:id="rId11" xr:uid="{16B8370C-655D-4F27-BD1C-3DEBDF8824DA}"/>
+    <hyperlink ref="R16" r:id="rId12" xr:uid="{A3AD2B59-8F70-46C7-9DD3-618BD825C254}"/>
+    <hyperlink ref="R17" r:id="rId13" xr:uid="{AA190877-4F5D-481B-A13A-290FDB73C5F0}"/>
+    <hyperlink ref="R18" r:id="rId14" display="mailto:claudiarafaelav@hotmail.com" xr:uid="{CF44BEFF-5A69-42C2-A487-F1067A570948}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audiências: sync 2026-10-05 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A4A1CA0-8BE0-4755-AA35-59DABE595CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B983A487-7B73-4AA1-8492-92DD0928A756}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E26630DF-7025-4C67-9939-633F9CC7DFF4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F708F57B-CDFA-44D6-BDAB-F111C37C5FFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="222">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,379 +95,616 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Inicial - Presencial</t>
+  </si>
+  <si>
+    <t>0000477-55.2026.5.23.0031</t>
+  </si>
+  <si>
+    <t>Dipagro Ltda</t>
+  </si>
+  <si>
+    <t>Kleber Garcia Barbara</t>
+  </si>
+  <si>
+    <t>CÁCERES</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$             212.847,22</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Correspondente</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0001131-63.2026.5.23.0121</t>
+  </si>
+  <si>
+    <t>Inpasa Agroindustrial S/A.</t>
+  </si>
+  <si>
+    <t>Vanildes Souza De Santana</t>
+  </si>
+  <si>
+    <t>NOVA MUTUM</t>
+  </si>
+  <si>
+    <t>R$          3.691.382,47</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>BTF</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>https://trt23-jus-br.zoom.us/my/vtnovamutum ID da reunião: 525 746 4936 Senha de acesso: @Nm121</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0001133-71.2026.5.23.0076</t>
+  </si>
+  <si>
+    <t>Agropecuaria Infiniti Ltda.</t>
+  </si>
+  <si>
+    <t>Welison Vasconcelos Candido</t>
+  </si>
+  <si>
+    <t>PRIMAVERA DO LESTE</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>R$             200.038,28</t>
+  </si>
+  <si>
+    <t>RRU</t>
+  </si>
+  <si>
+    <t>https://trt23-jus-br.zoom.us/my/salanobres?pwd=NmdUWFBwaGtBZHpucTdWSFQyR2oxUT09 ID: 269 890 9821 Senha geral: Nobres1@</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0012362-43.2025.5.15.0122</t>
+  </si>
+  <si>
+    <t>Pilkington Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Raphael Decanio Amancio</t>
+  </si>
+  <si>
+    <t>SUMARÉ</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>R$               40.946,58</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/84993384241?pwd=5k1SoEXEWUkAMtV6ck51bpX3LIg8Yz.1</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1001555-22.2025.5.02.0020</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Giovanni Alessandro Ribeiro Ramos</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>20ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             878.026,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1001173-20.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Jose Roberto Lopes Da Silva</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             152.575,89</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>0001513-14.2026.5.18.0083</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Jose Madalena Justiniano</t>
+  </si>
+  <si>
+    <t>RIO VERDE</t>
+  </si>
+  <si>
+    <t>GO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$             100.441,80</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>https://trt18-jus-br.zoom.us/my/cejuscrioverde</t>
+  </si>
+  <si>
+    <t>1000694-21.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Rubens Bernardes Da Silva</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             278.000,00</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0100938-16.2026.5.01.0203</t>
+  </si>
+  <si>
+    <t>Bruno Do Nascimento Monteiro</t>
+  </si>
+  <si>
+    <t>DUQUE DE CAXIAS</t>
+  </si>
+  <si>
+    <t>RJ</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             612.615,41</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>https://trt1-jus-br.zoom.us/my/vtdc03?pwd=all4TmdCN01CRGliVlp5dkh6aTBBdz09</t>
+  </si>
+  <si>
+    <t>0012105-48.2026.5.15.0133</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Manoel Correia Dias</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>R$             568.813,56</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/82214057803?pwd=Yk9reERlOGxwRk1wVjE2cHYzN29sQT09</t>
+  </si>
+  <si>
+    <t>0010052-17.2026.5.15.0094</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Priscila Pereira De Medeiros</t>
+  </si>
+  <si>
+    <t>CAMPINAS</t>
+  </si>
+  <si>
+    <t>07ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Ação de Consignação em Pagamento</t>
+  </si>
+  <si>
+    <t>R$               17.118,32</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/4525285196?pwd=cG1ieCtlVVdHZERxcVRTM2lzSGt3dz09 ID da reunião: 452 528 5196 Senha de acesso: 702632</t>
+  </si>
+  <si>
+    <t>1001372-08.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Weslley Igor Antonio Lopes Dos Santos</t>
+  </si>
+  <si>
+    <t>RIBEIRÃO PIRES</t>
+  </si>
+  <si>
+    <t>R$               45.484,31</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>1000515-59.2026.5.02.0411</t>
+  </si>
+  <si>
+    <t>Cbc - Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Vinicius De Souza Franca</t>
+  </si>
+  <si>
+    <t>R$             282.024,58</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>1001486-48.2025.5.02.0421</t>
+  </si>
+  <si>
+    <t>3Corp Technology Infraestrutura De Telecom Ltda.</t>
+  </si>
+  <si>
+    <t>Gabriel Tavares Parreira De Paula</t>
+  </si>
+  <si>
+    <t>SANTANA DE PARNAÍBA</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             157.171,00</t>
+  </si>
+  <si>
+    <t>Grupo A2</t>
+  </si>
+  <si>
+    <t>NBG</t>
+  </si>
+  <si>
+    <t>0010223-72.2026.5.15.0126</t>
+  </si>
+  <si>
+    <t>Sofia Da Silva Assis</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>R$             176.547,57</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>GVM</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/86534999498?pwd=N3RZZXpkTE5laWxEREEvWjBVYVg0Zz09 ID da reunião: 865 3499 9498 Senha: 13579</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>0010976-96.2026.5.03.0147</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A</t>
+  </si>
+  <si>
+    <t>Marcio Rezende Fonseca</t>
+  </si>
+  <si>
+    <t>TRÊS CORAÇÕES</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$          1.435.000,00</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Matheus Pimenta Barros matheuspb26@live.com 35999092279</t>
+  </si>
+  <si>
+    <t>Perícia Técnica</t>
+  </si>
+  <si>
+    <t>0012829-61.2025.5.15.0109</t>
+  </si>
+  <si>
+    <t>Umberto Aparecido Lima</t>
+  </si>
+  <si>
+    <t>SOROCABA</t>
+  </si>
+  <si>
+    <t>R$             856.425,61</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>Iremos acompanhar</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>1000179-05.2020.5.02.0431</t>
+  </si>
+  <si>
+    <t>Jose Ricardo Silva</t>
+  </si>
+  <si>
+    <t>CEJUSC ABC</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$             151.781,01</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/81026971770?pwd=WlJ4VkMvUUhBa1QxWUN1eldWeFNKQT09 ID da reunião: 810 2697 1770 Senha de acesso: 820150</t>
+  </si>
+  <si>
+    <t>1001462-42.2026.5.02.0467</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Fernando Lopes Bento</t>
+  </si>
+  <si>
+    <t>SÃO BERNARDO DO CAMPO</t>
+  </si>
+  <si>
+    <t>R$               45.442,32</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Dra. Luciana França, (11) 96351-8524</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>1001687-31.2025.5.02.0521</t>
-  </si>
-  <si>
-    <t>Mahle Thermal And Fluid Systems Brazil Ltda.</t>
-  </si>
-  <si>
-    <t>Rafael De Oliveira Andrade</t>
-  </si>
-  <si>
-    <t>ARUJÁ</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             440.000,00</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>TLI</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/86789289821?pwd=hmNmYn6ZPr5UBUkTREU7WbLud20xkY.1 ID da reunião: 867 8928 9821 Senha de acesso: vtaruja01</t>
-  </si>
-  <si>
-    <t>1001571-25.2025.5.02.0521</t>
-  </si>
-  <si>
-    <t>R$               87.965,00</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/86826984343?pwd=vqkjCTDTofwYe3zhKsVzowS3Wcmu4J.1 ID da reunião: 868 2698 4343 Senha de acesso: vtaruja01</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001457-38.2025.5.02.0052</t>
-  </si>
-  <si>
-    <t>Mccann Erickson Publicidade Ltda.</t>
-  </si>
-  <si>
-    <t>Ministério Público Do Trabalho</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>52ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Ação Civil Pública</t>
-  </si>
-  <si>
-    <t>R$          3.655.206,00</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
-  </si>
-  <si>
-    <t>NBG</t>
+    <t>0010335-20.2026.5.15.0133</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Renato Jose Dias</t>
+  </si>
+  <si>
+    <t>R$             418.460,00</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/7871570572?pwd=KzBzUnVURkZwc0gxd21YU3pUWWhJQT09 ID da reunião: 787 157 0572 Senha de acesso: 674353</t>
+  </si>
+  <si>
+    <t>0010667-75.2026.5.03.0147</t>
+  </si>
+  <si>
+    <t>Julio Henrique Dionisio</t>
+  </si>
+  <si>
+    <t>R$             712.000,00</t>
+  </si>
+  <si>
+    <t>BBO</t>
+  </si>
+  <si>
+    <t>0010664-23.2026.5.03.0147</t>
+  </si>
+  <si>
+    <t>Breno Heleno Da Silva Mariano</t>
+  </si>
+  <si>
+    <t>R$             521.000,00</t>
+  </si>
+  <si>
+    <t>0010380-36.2026.5.03.0140</t>
+  </si>
+  <si>
+    <t>Sistenge Construções E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Alex Alves Da Silva Batista</t>
+  </si>
+  <si>
+    <t>CONTAGEM</t>
+  </si>
+  <si>
+    <t>R$             114.705,18</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt1.contagem</t>
+  </si>
+  <si>
+    <t>0012594-95.2025.5.15.0044</t>
+  </si>
+  <si>
+    <t>Alex Cruz De Souza</t>
+  </si>
+  <si>
+    <t>R$             292.000,00</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/83908187251?pwd=Ty9tcHNFb0pLZk5WQ0l2Y0V3ZHhhdz09</t>
+  </si>
+  <si>
+    <t>1001057-08.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Elizeu Luiz Freire</t>
+  </si>
+  <si>
+    <t>R$             158.737,00</t>
+  </si>
+  <si>
+    <t>0024006-50.2026.5.24.0072</t>
+  </si>
+  <si>
+    <t>Rio Paraná Energia S.A.</t>
+  </si>
+  <si>
+    <t>Edson Barbosa</t>
+  </si>
+  <si>
+    <t>TRÊS LAGOAS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>R$             192.773,33</t>
   </si>
   <si>
     <t>ECO</t>
   </si>
   <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000890-85.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Joel Marcos Jose De Souza</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             832.800,15</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>1001113-13.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Gustavo Souza Da Silva</t>
-  </si>
-  <si>
-    <t>RIBEIRÃO PIRES</t>
-  </si>
-  <si>
-    <t>R$             191.930,23</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>LMI</t>
-  </si>
-  <si>
-    <t>0010906-32.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>Fertilizantes Heringer S.A</t>
-  </si>
-  <si>
-    <t>Antonio Carlos Da Costa Oliveira</t>
-  </si>
-  <si>
-    <t>PAULÍNIA</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Conhecimento</t>
-  </si>
-  <si>
-    <t>R$             427.015,86</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>AAP</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>0016784-42.2026.5.16.0011</t>
-  </si>
-  <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Jorge De Oliveira Santos</t>
-  </si>
-  <si>
-    <t>BALSAS</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>R$               85.170,87</t>
-  </si>
-  <si>
-    <t>JRM</t>
-  </si>
-  <si>
-    <t>GVM</t>
-  </si>
-  <si>
-    <t>https://us02web.zoom.us/j/84680881845?pwd=2uHgFIbgHPhxy5JJEP3uHrbe96HPcI.1 ID da reunião: 846 8088 1845 Senha: 960717</t>
-  </si>
-  <si>
-    <t>0011220-26.2022.5.15.0084</t>
-  </si>
-  <si>
-    <t>Eleb Equipamentos Ltda.</t>
-  </si>
-  <si>
-    <t>Carlos Eduardo Da Silva</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>04ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>R$             296.615,60</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>0010579-44.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda</t>
-  </si>
-  <si>
-    <t>Danilo Alves Vieira Junior</t>
-  </si>
-  <si>
-    <t>PATROCÍNIO</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>R$               80.346,37</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
-  </si>
-  <si>
-    <t>1000805-11.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Luis Guilherme Da Silva</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             955.048,98</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Semipresencial</t>
-  </si>
-  <si>
-    <t>0011464-69.2025.5.15.0012</t>
-  </si>
-  <si>
-    <t>Rafael De Oliveira Silva</t>
-  </si>
-  <si>
-    <t>PIRACICABA</t>
-  </si>
-  <si>
-    <t>R$             112.641,97</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>JPE</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/88307820364?pwd=S2FSa2QyaUQvZVBqRThqT25PeFNXQT09 ID da reunião: 88307820364 Senha de acesso: 277454</t>
-  </si>
-  <si>
-    <t>0011050-05.2025.5.15.0131</t>
-  </si>
-  <si>
-    <t>Aderson Jose Ferreira</t>
-  </si>
-  <si>
-    <t>R$               65.358,00</t>
-  </si>
-  <si>
-    <t>0010938-37.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>Israel Leandro Firmino Da Silva</t>
-  </si>
-  <si>
-    <t>R$             241.555,32</t>
-  </si>
-  <si>
-    <t>0000310-55.2026.5.09.0022</t>
-  </si>
-  <si>
-    <t>Rhian Carlos Dos Santos Rosa</t>
-  </si>
-  <si>
-    <t>PARANAGUÁ</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>R$               77.625,00</t>
-  </si>
-  <si>
-    <t>BBO</t>
-  </si>
-  <si>
-    <t>https://url.trt9.jus.br/tcxf3 ID da reunião: 84009977944 Senha de acesso: j4DeUgYBbf</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Presencial</t>
-  </si>
-  <si>
-    <t>0010945-29.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>Almir Rogerio Barbosa Da Silva</t>
-  </si>
-  <si>
-    <t>R$          1.139.691,67</t>
-  </si>
-  <si>
-    <t>Audiência Una- Telepresencial</t>
-  </si>
-  <si>
-    <t>1001294-49.2026.5.02.0464</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Deivmayk Aragao Dos Santos</t>
-  </si>
-  <si>
-    <t>SÃO BERNARDO DO CAMPO</t>
-  </si>
-  <si>
-    <t>R$               13.854,40</t>
-  </si>
-  <si>
-    <t>VRO</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/88393016008?pwd=TqCbvr2qbyfEpGCVS8ebEjSzAZFmrj.1</t>
+    <t>0011493-69.2022.5.15.0095</t>
+  </si>
+  <si>
+    <t>Jose Roberto Francisco</t>
+  </si>
+  <si>
+    <t>Execução</t>
+  </si>
+  <si>
+    <t>R$             157.477,74</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/89925839124?pwd=HehXMRH0LyTAyjb9t6axbYz7RHoBqz.1</t>
   </si>
 </sst>
 </file>
@@ -945,8 +1182,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B498F49-C313-495C-B427-786E56BC4DA7}">
-  <dimension ref="A1:R17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{012C189B-2E60-4599-964A-781DD785386B}">
+  <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
@@ -1005,12 +1242,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>101949</v>
+        <v>106670</v>
       </c>
       <c r="B2" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C2" s="6">
         <v>0.34027777777777779</v>
@@ -1057,34 +1294,34 @@
       <c r="Q2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>101858</v>
+        <v>106002</v>
       </c>
       <c r="B3" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C3" s="6">
-        <v>0.35416666666666669</v>
+        <v>0.34375</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>23</v>
@@ -1102,107 +1339,107 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>102088</v>
+        <v>105723</v>
       </c>
       <c r="B4" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C4" s="6">
-        <v>0.3611111111111111</v>
+        <v>0.35069444444444442</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>25</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="R4" s="7" t="s">
-        <v>47</v>
+        <v>40</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
-        <v>104972</v>
+        <v>101761</v>
       </c>
       <c r="B5" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3611111111111111</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>25</v>
@@ -1214,54 +1451,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>47</v>
+        <v>59</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>105685</v>
+        <v>104087</v>
       </c>
       <c r="B6" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C6" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J6" s="7" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1270,54 +1507,54 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>105358</v>
+        <v>105336</v>
       </c>
       <c r="B7" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C7" s="6">
-        <v>0.41666666666666669</v>
+        <v>0.39930555555555558</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J7" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>26</v>
@@ -1326,54 +1563,54 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="216.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>105337</v>
+        <v>105773</v>
       </c>
       <c r="B8" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C8" s="6">
-        <v>0.4375</v>
+        <v>0.40277777777777779</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1382,54 +1619,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="O8" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>88925</v>
+        <v>104747</v>
       </c>
       <c r="B9" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C9" s="6">
-        <v>0.4375</v>
+        <v>0.4236111111111111</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1438,54 +1675,54 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>105082</v>
+        <v>105434</v>
       </c>
       <c r="B10" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C10" s="6">
-        <v>0.45833333333333331</v>
+        <v>0.4236111111111111</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>24</v>
+        <v>102</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
@@ -1494,51 +1731,51 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="R10" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>104859</v>
+        <v>106022</v>
       </c>
       <c r="B11" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C11" s="6">
-        <v>0.46180555555555558</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>25</v>
@@ -1550,110 +1787,110 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O11" s="7" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>47</v>
+        <v>111</v>
+      </c>
+      <c r="R11" s="8" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>101549</v>
+        <v>103770</v>
       </c>
       <c r="B12" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C12" s="6">
-        <v>0.5</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>69</v>
+        <v>117</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>25</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>26</v>
+        <v>118</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="R12" s="8" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>105027</v>
+        <v>106134</v>
       </c>
       <c r="B13" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C13" s="6">
-        <v>0.56944444444444442</v>
+        <v>0.4375</v>
       </c>
       <c r="D13" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J13" s="7" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>26</v>
@@ -1662,54 +1899,54 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>105340</v>
+        <v>104671</v>
       </c>
       <c r="B14" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C14" s="6">
-        <v>0.57013888888888886</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>23</v>
-      </c>
       <c r="J14" s="7" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>26</v>
@@ -1718,54 +1955,54 @@
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>104852</v>
+        <v>102963</v>
       </c>
       <c r="B15" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C15" s="6">
-        <v>0.58333333333333337</v>
+        <v>0.5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>75</v>
+        <v>134</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>66</v>
+        <v>136</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>127</v>
+        <v>57</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>69</v>
+        <v>139</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>26</v>
@@ -1774,54 +2011,54 @@
         <v>27</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>72</v>
+        <v>141</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>102</v>
+        <v>142</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="R15" s="8" t="s">
-        <v>130</v>
+        <v>142</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>105374</v>
+        <v>104206</v>
       </c>
       <c r="B16" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C16" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.52777777777777779</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>131</v>
+        <v>33</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>68</v>
+        <v>145</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>26</v>
@@ -1830,54 +2067,54 @@
         <v>27</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="O16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>84</v>
+        <v>147</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="R16" s="7" t="s">
-        <v>47</v>
+        <v>148</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>149</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
-        <v>105793</v>
+        <v>106041</v>
       </c>
       <c r="B17" s="5">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="C17" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>23</v>
+        <v>155</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>91</v>
+        <v>156</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>26</v>
@@ -1886,30 +2123,655 @@
         <v>27</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="O17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>103165</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>76146</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.5444444444444444</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R19" s="8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>106007</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="O20" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="P17" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="Q17" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="R17" s="8" t="s">
-        <v>142</v>
+      <c r="P20" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="R20" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>104554</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R21" s="8" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>105356</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q22" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="R22" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>105355</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="O23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="R23" s="8" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>104705</v>
+      </c>
+      <c r="B24" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.58750000000000002</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R24" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>103161</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="R25" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>105230</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q26" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="R26" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>103734</v>
+      </c>
+      <c r="B27" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0.65972222222222221</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N27" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="O27" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="P27" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>96644</v>
+      </c>
+      <c r="B28" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C28" s="6">
+        <v>0.66111111111111109</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N28" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="O28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P28" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q28" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="R28" s="8" t="s">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" display="https://trt2-jus-br.zoom.us/j/86789289821?pwd=hmNmYn6ZPr5UBUkTREU7WbLud20xkY.1%20ID%20da%20reunião:%20867%208928%209821%20Senha%20de%20acesso:%20vtaruja01" xr:uid="{E7FFCD97-24DB-43AB-9395-57087B28248F}"/>
-    <hyperlink ref="R3" r:id="rId2" display="https://trt2-jus-br.zoom.us/j/86826984343?pwd=vqkjCTDTofwYe3zhKsVzowS3Wcmu4J.1%20ID%20da%20reunião:%20868%202698%204343%20Senha%20de%20acesso:%20vtaruja01" xr:uid="{80454755-258F-43E6-A9D4-10DF4AD92B37}"/>
-    <hyperlink ref="R8" r:id="rId3" display="https://us02web.zoom.us/j/84680881845?pwd=2uHgFIbgHPhxy5JJEP3uHrbe96HPcI.1%20ID%20da%20reunião:%20846%208088%201845%20Senha:%20960717" xr:uid="{8AAD73CB-208E-436C-BB5A-24992423B349}"/>
-    <hyperlink ref="R10" r:id="rId4" xr:uid="{96DEECF1-4D10-4741-8773-D9C26F477D09}"/>
-    <hyperlink ref="R12" r:id="rId5" display="https://trt15-jus-br.zoom.us/j/88307820364?pwd=S2FSa2QyaUQvZVBqRThqT25PeFNXQT09%20ID%20da%20reunião:%2088307820364%20Senha%20de%20acesso:%20277454" xr:uid="{2E307451-92D6-4ABF-9243-28C015D7F693}"/>
-    <hyperlink ref="R15" r:id="rId6" xr:uid="{B64BBBFC-C518-451D-A498-513B0DEED800}"/>
-    <hyperlink ref="R17" r:id="rId7" xr:uid="{D9FE39BB-B3B9-46E2-9419-191D17FE1C87}"/>
+    <hyperlink ref="R3" r:id="rId1" xr:uid="{9145FE9B-8F7D-4B88-B76E-C894EF6F7E6C}"/>
+    <hyperlink ref="R4" r:id="rId2" display="https://trt23-jus-br.zoom.us/my/salanobres?pwd=NmdUWFBwaGtBZHpucTdWSFQyR2oxUT09" xr:uid="{F6FC0837-52FC-4D2A-8BE7-925D92285230}"/>
+    <hyperlink ref="R5" r:id="rId3" xr:uid="{EAF25487-F171-4499-BCD6-E01F1F87CEEB}"/>
+    <hyperlink ref="R8" r:id="rId4" xr:uid="{E3F8ABC5-B8A5-4735-848E-07FF20AADDE0}"/>
+    <hyperlink ref="R10" r:id="rId5" xr:uid="{E7D8DE9F-E84E-4EEA-BDD4-D52F4DC82248}"/>
+    <hyperlink ref="R11" r:id="rId6" xr:uid="{0372A527-6999-4904-B1B1-7A43C807ADA5}"/>
+    <hyperlink ref="R12" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/4525285196?pwd=cG1ieCtlVVdHZERxcVRTM2lzSGt3dz09%20ID%20da%20reunião:%20452%20528%205196%20Senha%20de%20acesso:%20702632" xr:uid="{61BAF5AF-4A3D-4EC6-A380-749DB18C1040}"/>
+    <hyperlink ref="R16" r:id="rId8" display="https://trt15-jus-br.zoom.us/j/86534999498?pwd=N3RZZXpkTE5laWxEREEvWjBVYVg0Zz09%20ID%20da%20reunião:%20865%203499%209498%20Senha:%2013579" xr:uid="{8576BC53-723C-4BBA-A067-698A9A809409}"/>
+    <hyperlink ref="R17" r:id="rId9" display="mailto:matheuspb26@live.com" xr:uid="{D2BB5679-0297-4404-B611-B94B28CF6974}"/>
+    <hyperlink ref="R19" r:id="rId10" display="https://trt2-jus-br.zoom.us/j/81026971770?pwd=WlJ4VkMvUUhBa1QxWUN1eldWeFNKQT09%20ID%20da%20reunião:%20810%202697%201770%20Senha%20de%20acesso:%20820150" xr:uid="{D6F1EA05-92C1-4A4E-AF5E-73A29FE5501C}"/>
+    <hyperlink ref="R21" r:id="rId11" display="https://trt15-jus-br.zoom.us/j/7871570572?pwd=KzBzUnVURkZwc0gxd21YU3pUWWhJQT09%20ID%20da%20reunião:%20787%20157%200572%20Senha%20de%20acesso:%20674353" xr:uid="{2364E6AF-97A0-4AEB-B8F5-FDB625C0747E}"/>
+    <hyperlink ref="R22" r:id="rId12" display="mailto:matheuspb26@live.com" xr:uid="{1E125AA0-242B-4E78-A958-7CAF776E5B63}"/>
+    <hyperlink ref="R23" r:id="rId13" display="mailto:matheuspb26@live.com" xr:uid="{DC503282-8A2D-4497-80CB-09659BD83F7C}"/>
+    <hyperlink ref="R24" r:id="rId14" xr:uid="{C9A4610A-B736-450F-AC71-6739F0C3ACE7}"/>
+    <hyperlink ref="R25" r:id="rId15" xr:uid="{B4D0ED84-C030-4D8F-B51A-DE31A3EE6F96}"/>
+    <hyperlink ref="R28" r:id="rId16" xr:uid="{9B47D63E-A368-4AE6-A9BF-4488A381A077}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-10-13 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{63C06E1E-C725-41C3-8C62-2E541EE4A9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{931DB7A8-D032-4F01-85F3-02334A245A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9D782BEA-4731-472A-B1C4-FBA531634020}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0D68274D-A94B-4137-BA4F-C6EB2A6D96FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="188">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,142 +95,514 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>1001831-47.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Rodrigo Ventura Da Silva</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$             184.477,10</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0012499-18.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Artur Alberto Chieregatti Junior</t>
+  </si>
+  <si>
+    <t>MOGI GUAÇU</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             345.912,99</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Correspondente - Ana Carolina Teresani</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>0011449-03.2026.5.03.0044</t>
-  </si>
-  <si>
-    <t>Syngenta Seeds Ltda.</t>
-  </si>
-  <si>
-    <t>Rafael Vidal Da Silva</t>
-  </si>
-  <si>
-    <t>UBERLÂNDIA</t>
+    <t>0000573-66.2026.5.09.0126</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações</t>
+  </si>
+  <si>
+    <t>Osnilto Teodoro Dos Santos</t>
+  </si>
+  <si>
+    <t>PALMAS</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>R$             576.500,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/as9c5 ID da Reunião: 87076063050 Senha: 8rWy03lvY1</t>
+  </si>
+  <si>
+    <t>0011080-53.2026.5.15.0083</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Leandro Borduchi</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             115.000,00</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>0011089-15.2026.5.15.0083</t>
+  </si>
+  <si>
+    <t>Gilberto Anderson Pereira</t>
+  </si>
+  <si>
+    <t>R$             172.500,00</t>
+  </si>
+  <si>
+    <t>BCF</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Semipresencial</t>
+  </si>
+  <si>
+    <t>0024705-94.2026.5.24.0022</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Monteverde</t>
+  </si>
+  <si>
+    <t>Gabriel Florenciano Da Silva</t>
+  </si>
+  <si>
+    <t>DOURADOS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             245.432,47</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/my/trt24douvt2sala1</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1000798-23.2026.5.02.0075</t>
+  </si>
+  <si>
+    <t>T4F Entretenimento S.A</t>
+  </si>
+  <si>
+    <t>Diego Monteiro Santos Prado</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>75ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$             166.195,36</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>1001909-41.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Antonio Idalbancir Dias Coelho</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             487.482,55</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0010209-93.2025.5.15.0071</t>
+  </si>
+  <si>
+    <t>Archimedes Barbosa Siqueira</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>R$             125.701,08</t>
+  </si>
+  <si>
+    <t>1000724-56.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Wilson Aparecido Sant Ana</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               79.500,00</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>0011122-47.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Joao Paulo De Oliveira Faria</t>
+  </si>
+  <si>
+    <t>PATROCÍNIO</t>
   </si>
   <si>
     <t>MG</t>
   </si>
   <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$               78.008,71</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
+    <t>R$             122.727,28</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
+  </si>
+  <si>
+    <t>1000557-62.2026.5.02.0006</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Mario Roberto De Lima</t>
+  </si>
+  <si>
+    <t>06ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          1.582.455,98</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>0011123-32.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Matheus Finetti Zanardo</t>
+  </si>
+  <si>
+    <t>1001053-77.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Graziele Novais Dos Santos</t>
+  </si>
+  <si>
+    <t>R$             200.175,46</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>1002323-73.2025.5.02.0431</t>
+  </si>
+  <si>
+    <t>Higor Dos Santos</t>
+  </si>
+  <si>
+    <t>R$             582.095,16</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010613-19.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Salitre Fetilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Maria Izabel Amorim Costa</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$               34.420,70</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Semipresencial</t>
+  </si>
+  <si>
+    <t>0011790-44.2024.5.15.0083</t>
+  </si>
+  <si>
+    <t>Kennedy Carvalho Lucas</t>
+  </si>
+  <si>
+    <t>02ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal TRT</t>
+  </si>
+  <si>
+    <t>R$             147.500,00</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/launch/jc/86986668664 ID da reunião: 869 8666 8664 Senha: 410044</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0012495-75.2025.5.15.0093</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Eduardo Henrique Maia Carnauba</t>
+  </si>
+  <si>
+    <t>CAMPINAS</t>
+  </si>
+  <si>
+    <t>R$             596.014,50</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81469918489?pwd=NmNHNVdhSERvZHorOXRIdmJCWU5MQT09 ID da reunião: 814 6991 8489 Senha: 059291</t>
+  </si>
+  <si>
+    <t>0010133-49.2026.5.15.0131</t>
+  </si>
+  <si>
+    <t>Alex Gomes De Sousa</t>
+  </si>
+  <si>
+    <t>12ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             179.903,44</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/86534999498?pwd=N3RZZXpkTE5laWxEREEvWjBVYVg0Zz0</t>
+  </si>
+  <si>
+    <t>0010841-17.2026.5.15.0126</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Claudinei Dos Santos</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>R$               38.195,57</t>
+  </si>
+  <si>
+    <t>JPL</t>
   </si>
   <si>
     <t>GVM</t>
   </si>
   <si>
-    <t>https://trt3-jus-br.zoom.us/j/81879397512?pwd=VdlZu0aH7a5vBp2FDhtwnWTDjaiSns.1</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001319-56.2026.5.02.0466</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Everton Aparecido Dos Santos</t>
-  </si>
-  <si>
-    <t>SÃO BERNARDO DO CAMPO</t>
-  </si>
-  <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>06ª VARA DO TRABALHO</t>
+    <t>https://trt15-jus-br.zoom.us/j/83059104477?pwd=h7VDkteaYgzZ4FIU9CoepcQo5ErUHA.1 ID da reunião: 830 5910 4477 Senha: 005974</t>
+  </si>
+  <si>
+    <t>0012011-90.2025.5.15.0083</t>
+  </si>
+  <si>
+    <t>Maria Fernanda Vila Nova Marson Schuller</t>
   </si>
   <si>
     <t>Inicial</t>
   </si>
   <si>
-    <t>R$               64.827,60</t>
-  </si>
-  <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>TLI</t>
-  </si>
-  <si>
-    <t>Presencial | Advogada - Dra. Luciana França, (11) 96351-8524</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>1001656-47.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Marcos Rogerio Romero</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>R$          1.346.621,89</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>1001394-66.2026.5.02.0411</t>
-  </si>
-  <si>
-    <t>Companhia Brasileira De Cartuchos</t>
-  </si>
-  <si>
-    <t>Luciano Rodrigues Da Costa</t>
-  </si>
-  <si>
-    <t>RIBEIRÃO PIRES</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$               31.230,99</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>LMI</t>
+    <t>R$             149.105,07</t>
+  </si>
+  <si>
+    <t>0011989-36.2024.5.15.0093</t>
+  </si>
+  <si>
+    <t>Gregory Ragosta Cassiano De Souza</t>
+  </si>
+  <si>
+    <t>05ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$          1.066.473,00</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88116222157?pwd=oFe1QBH0rStbUhO7ngHqYzIDE9abay.1</t>
+  </si>
+  <si>
+    <t>0010618-84.2026.5.15.0087</t>
+  </si>
+  <si>
+    <t>Rogerio Cordeiro</t>
+  </si>
+  <si>
+    <t>R$          1.150.491,32</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/81792542599?pwd=dWt0TnU2UXVUYXdKTU1CU2gzUTVZQT09 ID da reunião: 817 9254 2599 Senha: 692443</t>
+  </si>
+  <si>
+    <t>0001673-47.2025.5.09.0011</t>
+  </si>
+  <si>
+    <t>Jose Aparecido Dos Santos Wermer</t>
+  </si>
+  <si>
+    <t>CURITIBA</t>
+  </si>
+  <si>
+    <t>11ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             303.594,35</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>1000994-20.2025.5.02.0433</t>
+  </si>
+  <si>
+    <t>Sidinei De Souza Oliveira</t>
+  </si>
+  <si>
+    <t>R$             400.000,00</t>
+  </si>
+  <si>
+    <t>0012474-76.2025.5.15.0133</t>
+  </si>
+  <si>
+    <t>Marcelo Luiz Teixeira</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>Produção Antecipada de Prova</t>
+  </si>
+  <si>
+    <t>R$                    500,00</t>
   </si>
 </sst>
 </file>
@@ -708,8 +1080,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687A6575-026E-42C4-A52B-49D3364B11A4}">
-  <dimension ref="A1:R5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49ED9DFC-A4C8-407F-936A-93E44AF2209F}">
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
@@ -768,12 +1140,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>105829</v>
+        <v>106140</v>
       </c>
       <c r="B2" s="5">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="C2" s="6">
         <v>0.375</v>
@@ -818,45 +1190,45 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" s="8" t="s">
         <v>31</v>
       </c>
+      <c r="R2" s="7" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>105792</v>
+        <v>99850</v>
       </c>
       <c r="B3" s="5">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="C3" s="6">
-        <v>0.44791666666666669</v>
+        <v>0.375</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -865,10 +1237,10 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="O3" s="7" t="s">
-        <v>29</v>
       </c>
       <c r="P3" s="7" t="s">
         <v>41</v>
@@ -877,42 +1249,42 @@
         <v>42</v>
       </c>
       <c r="R3" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>105023</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>106139</v>
-      </c>
-      <c r="B4" s="5">
-        <v>46304</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0.49305555555555558</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>37</v>
-      </c>
       <c r="J4" s="7" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -921,54 +1293,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="R4" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="Q4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>105032</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="R4" s="7" t="s">
+      <c r="F5" s="7" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>106211</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46304</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>60</v>
-      </c>
       <c r="K5" s="7" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -977,24 +1349,1267 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="P5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>105033</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.3923611111111111</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="F6" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="Q5" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="R5" s="7" t="s">
+      <c r="H6" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>104774</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C7" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="R7" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>105223</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>106263</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>99950</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>104771</v>
+      </c>
+      <c r="B11" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.4201388888888889</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>106063</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="R12" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>104667</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>106100</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="R14" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>105182</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.47222222222222221</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>103551</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.4861111111111111</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>105174</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>98816</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>55</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="R18" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>103490</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="R19" s="8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>103858</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R20" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>105111</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="R21" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>102063</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q22" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="R22" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>104088</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="O23" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="R23" s="8" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>104804</v>
+      </c>
+      <c r="B24" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.61805555555555558</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q24" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="R24" s="8" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="96.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>103582</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="R25" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>101364</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q26" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R26" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>104114</v>
+      </c>
+      <c r="B27" s="5">
+        <v>46308</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N27" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="O27" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="P27" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="R27" s="8" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" xr:uid="{C89B7E5D-4D81-4675-BD34-71D697924965}"/>
+    <hyperlink ref="R4" r:id="rId1" xr:uid="{310473BB-B8CD-4DD8-8B8D-401BBE0BFB8D}"/>
+    <hyperlink ref="R7" r:id="rId2" xr:uid="{ADC369A2-DDBB-427A-8792-139A5490DAEB}"/>
+    <hyperlink ref="R12" r:id="rId3" xr:uid="{F5A0AD32-BCCB-4E63-97FF-CEEEA8E86AAB}"/>
+    <hyperlink ref="R14" r:id="rId4" xr:uid="{7C10BA1F-B68E-4AFB-8778-6CC1142B93A2}"/>
+    <hyperlink ref="R17" r:id="rId5" xr:uid="{96BB691E-FBB2-4A4D-8513-4B1CF0268199}"/>
+    <hyperlink ref="R18" r:id="rId6" xr:uid="{1B78F597-5AE0-4860-A993-4CEB4BF32486}"/>
+    <hyperlink ref="R19" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/81469918489?pwd=NmNHNVdhSERvZHorOXRIdmJCWU5MQT09%20ID%20da%20reunião:%20814%206991%208489%20Senha:%20059291" xr:uid="{54D7A758-1309-469C-B422-56A798998E2F}"/>
+    <hyperlink ref="R20" r:id="rId8" xr:uid="{A9451B6D-1FCD-4B0B-94BB-C1F1BD247588}"/>
+    <hyperlink ref="R21" r:id="rId9" display="https://trt15-jus-br.zoom.us/j/83059104477?pwd=h7VDkteaYgzZ4FIU9CoepcQo5ErUHA.1%20ID%20da%20reunião:%20830%205910%204477%20Senha:%20005974" xr:uid="{9A116859-DC0B-4508-A064-B9E8DFF3843D}"/>
+    <hyperlink ref="R23" r:id="rId10" xr:uid="{4CB3E34E-FC69-47E4-BCF5-7FE5E6492AD6}"/>
+    <hyperlink ref="R24" r:id="rId11" display="https://trt15-jus-br.zoom.us/j/81792542599?pwd=dWt0TnU2UXVUYXdKTU1CU2gzUTVZQT09%20ID%20da%20reunião:%20817%209254%202599%20Senha:%20692443" xr:uid="{59384DEE-FAC9-4D0C-B7ED-78FE9ABEF94D}"/>
+    <hyperlink ref="R27" r:id="rId12" xr:uid="{40C6B6EB-5908-4C50-8E3D-9AC500DFFA27}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-10-14 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{931DB7A8-D032-4F01-85F3-02334A245A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45815E3B-F138-4721-B61D-892D22D06F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0D68274D-A94B-4137-BA4F-C6EB2A6D96FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3CB4E181-A3C7-4A68-81AE-A573CE9FE004}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="227">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,514 +95,631 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010728-44.2023.5.15.0037</t>
+  </si>
+  <si>
+    <t>Ouroeste Bioenergia Ltda.</t>
+  </si>
+  <si>
+    <t>Grazielly Olivia Venancio</t>
+  </si>
+  <si>
+    <t>FERNANDÓPOLIS</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>Liquidação</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$             333.194,18</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>LWP</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/88415253122?pwd=QzlTNmxwdWpEeGVFZmdwM0lDUFJ4Zz09 ID da reunião: 884 1525 3122 Senha de acesso: 510562</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010947-07.2026.5.03.0063</t>
+  </si>
+  <si>
+    <t>Syngenta Seeds Ltda</t>
+  </si>
+  <si>
+    <t>Cleiton Baltazar De Souza</t>
+  </si>
+  <si>
+    <t>ITUIUTABA</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>R$               39.600,00</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/j/85042016732</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Presencial</t>
   </si>
   <si>
-    <t>1001831-47.2026.5.02.0431</t>
+    <t>1001918-91.2026.5.02.0434</t>
   </si>
   <si>
     <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
   </si>
   <si>
-    <t>Rodrigo Ventura Da Silva</t>
+    <t>Erik Da Silva Prado</t>
   </si>
   <si>
     <t>SANTO ANDRÉ</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             184.477,10</t>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             272.182,03</t>
   </si>
   <si>
     <t>Grupo B1</t>
   </si>
   <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0010948-89.2026.5.03.0063</t>
+  </si>
+  <si>
+    <t>Luis Claudio Da Silva</t>
+  </si>
+  <si>
+    <t>R$             170.500,00</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TST - Presencial</t>
+  </si>
+  <si>
+    <t>1001280-40.2022.5.02.0065</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Silvio Luiz Rocca Ribeiro</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>01ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$          2.512.192,00</t>
+  </si>
+  <si>
+    <t>Grupo C</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>https://tst-jus-br.zoom.us/my/setr1</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011423-72.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Pilkington Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Richard Lopes Da Silva</t>
+  </si>
+  <si>
+    <t>CAÇAPAVA</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               56.759,19</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/86212862282?pwd=N2N4b3NobCtXbUxsODdmSXFlMjVCQT09 ID da reunião: 862 1286 2282 Senha: 498067</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
+  </si>
+  <si>
+    <t>0025858-49.2025.5.24.0071</t>
+  </si>
+  <si>
+    <t>Rio Paraná Energia S.A.</t>
+  </si>
+  <si>
+    <t>Orlando Homma De Souza</t>
+  </si>
+  <si>
+    <t>TRÊS LAGOAS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>02ª TURMA</t>
+  </si>
+  <si>
+    <t>R$               38.605,50</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>https://trt24-jus-br.zoom.us/j/84024327508?pwd=v3IAXTUTZyGmecL3g15WRYMaB8ufTj.1</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>1000470-81.2026.5.02.0467</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Nelson Luis Ribeiro</t>
+  </si>
+  <si>
+    <t>SÃO BERNARDO DO CAMPO</t>
+  </si>
+  <si>
+    <t>07ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             119.733,98</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Dra. Luciana França, (11) 96351-8524</t>
+  </si>
+  <si>
+    <t>0011832-75.2026.5.15.0131</t>
+  </si>
+  <si>
+    <t>Marcelo Jacome Da Costa</t>
+  </si>
+  <si>
+    <t>CAMPINAS</t>
+  </si>
+  <si>
+    <t>12ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               87.970,55</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/85453506049?pwd=Q0lIZFc3eS9kaGNJQ3N0cEIxdnBnZz09 ID da reunião: 854 5350 6049 Senha de acesso: 364 591</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1001356-43.2026.5.02.0059</t>
+  </si>
+  <si>
+    <t>Pedro Afonso Bioenergia Ltda</t>
+  </si>
+  <si>
+    <t>Lucas Villaca Ferreira De Oliveira</t>
+  </si>
+  <si>
+    <t>59ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$             122.575,93</t>
+  </si>
+  <si>
+    <t>BBO</t>
+  </si>
+  <si>
+    <t>1001581-08.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>Alex Dos Santos Silva</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               59.798,31</t>
+  </si>
+  <si>
     <t>JPE</t>
   </si>
   <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0012499-18.2024.5.15.0071</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Artur Alberto Chieregatti Junior</t>
-  </si>
-  <si>
-    <t>MOGI GUAÇU</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             345.912,99</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>Correspondente - Ana Carolina Teresani</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>0000573-66.2026.5.09.0126</t>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>0000919-74.2025.5.05.0122</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Eduardo Ferreira Brito</t>
+  </si>
+  <si>
+    <t>CANDEIAS</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>R$               26.714,27</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/j/81333809109?pwd=47akSzaeNwYTr7VDOZiMN5qQCeHjkO.1 ID da reunião: 813 3380 9109 Senha de acesso: 470307</t>
+  </si>
+  <si>
+    <t>0010500-04.2018.5.15.0083</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Alexandre Aparecido De Oliveira</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>CEJUSC TST</t>
+  </si>
+  <si>
+    <t>Recursal TST</t>
+  </si>
+  <si>
+    <t>R$               40.000,00</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>bit.ly/Cejusc2026</t>
+  </si>
+  <si>
+    <t>1001410-24.2025.5.02.0421</t>
+  </si>
+  <si>
+    <t>3Corp Technology Infraestrutura De Telecom Ltda.</t>
+  </si>
+  <si>
+    <t>Guilherme Arnaldo Da Silva Tomaz</t>
+  </si>
+  <si>
+    <t>SANTANA DE PARNAÍBA</t>
+  </si>
+  <si>
+    <t>R$             142.871,81</t>
+  </si>
+  <si>
+    <t>Grupo A2</t>
+  </si>
+  <si>
+    <t>NBG</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0010950-84.2025.5.15.0152</t>
+  </si>
+  <si>
+    <t>Sistenge Construções E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Angelo Roberto Soares Alves</t>
+  </si>
+  <si>
+    <t>HORTOLÂNDIA</t>
+  </si>
+  <si>
+    <t>R$               12.065,80</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>1000533-11.2026.5.02.0434</t>
+  </si>
+  <si>
+    <t>Valmir Eleodorio Da Silva</t>
+  </si>
+  <si>
+    <t>R$             126.726,60</t>
+  </si>
+  <si>
+    <t>0010123-63.2026.5.03.0058</t>
+  </si>
+  <si>
+    <t>Fertilizantes Heringer S.A.</t>
+  </si>
+  <si>
+    <t>Nei Ponciano</t>
+  </si>
+  <si>
+    <t>FORMIGA</t>
+  </si>
+  <si>
+    <t>R$             439.815,20</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt1formiga</t>
+  </si>
+  <si>
+    <t>1000973-20.2026.5.02.0462</t>
+  </si>
+  <si>
+    <t>Sonia Soares Almeida</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             191.275,42</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>0010841-91.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Juliano Roberto Ferreira</t>
+  </si>
+  <si>
+    <t>PATROCÍNIO</t>
+  </si>
+  <si>
+    <t>R$          1.218.035,77</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
+  </si>
+  <si>
+    <t>0000687-77.2025.5.12.0054</t>
+  </si>
+  <si>
+    <t>Wickbold &amp; Nosso Pão Indústrias Alimentícias Ltda</t>
+  </si>
+  <si>
+    <t>Jailson Cardoso</t>
+  </si>
+  <si>
+    <t>03ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal TRT</t>
+  </si>
+  <si>
+    <t>R$             474.999,97</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>link pendente</t>
+  </si>
+  <si>
+    <t>0011127-48.2025.5.15.0152</t>
+  </si>
+  <si>
+    <t>Dell Computadores Do Brasil Ltda</t>
+  </si>
+  <si>
+    <t>Izabela Macena Serrano</t>
+  </si>
+  <si>
+    <t>R$                 4.092,39</t>
+  </si>
+  <si>
+    <t>AAP</t>
+  </si>
+  <si>
+    <t>JPL</t>
+  </si>
+  <si>
+    <t>0000787-46.2026.5.23.0036</t>
+  </si>
+  <si>
+    <t>Inpasa Agroindustrial S/A.</t>
+  </si>
+  <si>
+    <t>Washington Luis Arruda Ribeiro</t>
+  </si>
+  <si>
+    <t>SINOP</t>
+  </si>
+  <si>
+    <t>MT</t>
+  </si>
+  <si>
+    <t>R$             327.566,94</t>
+  </si>
+  <si>
+    <t>BTF</t>
+  </si>
+  <si>
+    <t>https://trt23-jus-br.zoom.us/j/81753761549?pwd=NYkhI185ab9wC4FuLVDoNH2aVuBPb3.1 ID da reunião: 817 5376 1549 Senha: @VTSinop1</t>
+  </si>
+  <si>
+    <t>0000008-81.2026.5.09.0133</t>
   </si>
   <si>
     <t>Companhia Act De Participações E Companhia Aix De Participações</t>
   </si>
   <si>
-    <t>Osnilto Teodoro Dos Santos</t>
-  </si>
-  <si>
-    <t>PALMAS</t>
+    <t>Marcelo Aparecido Ramos</t>
+  </si>
+  <si>
+    <t>APUCARANA</t>
   </si>
   <si>
     <t>PR</t>
   </si>
   <si>
-    <t>R$             576.500,00</t>
-  </si>
-  <si>
-    <t>Grupo C</t>
-  </si>
-  <si>
-    <t>ECO</t>
+    <t>06ª TURMA</t>
+  </si>
+  <si>
+    <t>R$               60.000,00</t>
+  </si>
+  <si>
+    <t>RCF</t>
   </si>
   <si>
     <t>VSI</t>
   </si>
   <si>
-    <t>https://url.trt9.jus.br/as9c5 ID da Reunião: 87076063050 Senha: 8rWy03lvY1</t>
-  </si>
-  <si>
-    <t>0011080-53.2026.5.15.0083</t>
-  </si>
-  <si>
-    <t>Embraer S.A.</t>
-  </si>
-  <si>
-    <t>Leandro Borduchi</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             115.000,00</t>
-  </si>
-  <si>
-    <t>Grupo B2</t>
-  </si>
-  <si>
-    <t>VCR</t>
-  </si>
-  <si>
-    <t>0011089-15.2026.5.15.0083</t>
-  </si>
-  <si>
-    <t>Gilberto Anderson Pereira</t>
-  </si>
-  <si>
-    <t>R$             172.500,00</t>
-  </si>
-  <si>
-    <t>BCF</t>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Semipresencial</t>
-  </si>
-  <si>
-    <t>0024705-94.2026.5.24.0022</t>
-  </si>
-  <si>
-    <t>Moema Bioenergia S.A. - Monteverde</t>
-  </si>
-  <si>
-    <t>Gabriel Florenciano Da Silva</t>
-  </si>
-  <si>
-    <t>DOURADOS</t>
-  </si>
-  <si>
-    <t>MS</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             245.432,47</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>https://trt24-jus-br.zoom.us/my/trt24douvt2sala1</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1000798-23.2026.5.02.0075</t>
-  </si>
-  <si>
-    <t>T4F Entretenimento S.A</t>
-  </si>
-  <si>
-    <t>Diego Monteiro Santos Prado</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>75ª VARA DO TRABALHO</t>
+    <t>https://trt9-jus-br.zoom.us/j/82898229693?pwd=WFk5UElWZGpDYjR0a1hTa2xwSHNjdz09 ID reunião : 828 9822 9693 Senha de acesso: 434474</t>
+  </si>
+  <si>
+    <t>0011501-63.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Luciano Da Silva Duarte</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>R$             790.758,96</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1 ID da reunião: 885 4267 2682 Senha de acesso: 050728</t>
+  </si>
+  <si>
+    <t>0011702-56.2025.5.15.0152</t>
+  </si>
+  <si>
+    <t>Dell Computadores Do Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Gabriela Bueno Constantino</t>
+  </si>
+  <si>
+    <t>R$             102.584,06</t>
+  </si>
+  <si>
+    <t>0010649-96.2026.5.15.0025</t>
+  </si>
+  <si>
+    <t>Cesar Roberto De Souza Neto</t>
+  </si>
+  <si>
+    <t>BOTUCATU</t>
+  </si>
+  <si>
+    <t>R$             190.723,91</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/87539096808?pwd=ZG9OblpFcVRDVnFiNUdrZEdkazkzQT09</t>
+  </si>
+  <si>
+    <t>0011533-70.2025.5.15.0087</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Angelo Marcos De Oliveira</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
   </si>
   <si>
     <t>1ª Instância</t>
   </si>
   <si>
-    <t>R$             166.195,36</t>
-  </si>
-  <si>
-    <t>Grupo B3</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>1001909-41.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Antonio Idalbancir Dias Coelho</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             487.482,55</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0010209-93.2025.5.15.0071</t>
-  </si>
-  <si>
-    <t>Archimedes Barbosa Siqueira</t>
-  </si>
-  <si>
-    <t>Central</t>
-  </si>
-  <si>
-    <t>R$             125.701,08</t>
-  </si>
-  <si>
-    <t>1000724-56.2026.5.02.0434</t>
-  </si>
-  <si>
-    <t>Wilson Aparecido Sant Ana</t>
-  </si>
-  <si>
-    <t>04ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$               79.500,00</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>0011122-47.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda</t>
-  </si>
-  <si>
-    <t>Joao Paulo De Oliveira Faria</t>
-  </si>
-  <si>
-    <t>PATROCÍNIO</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>R$             122.727,28</t>
-  </si>
-  <si>
-    <t>CAL</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
-  </si>
-  <si>
-    <t>1000557-62.2026.5.02.0006</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Mario Roberto De Lima</t>
-  </si>
-  <si>
-    <t>06ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          1.582.455,98</t>
-  </si>
-  <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>0011123-32.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>Matheus Finetti Zanardo</t>
-  </si>
-  <si>
-    <t>1001053-77.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Graziele Novais Dos Santos</t>
-  </si>
-  <si>
-    <t>R$             200.175,46</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>1002323-73.2025.5.02.0431</t>
-  </si>
-  <si>
-    <t>Higor Dos Santos</t>
-  </si>
-  <si>
-    <t>R$             582.095,16</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>0010613-19.2026.5.03.0080</t>
-  </si>
-  <si>
-    <t>Salitre Fetilizantes Ltda</t>
-  </si>
-  <si>
-    <t>Maria Izabel Amorim Costa</t>
-  </si>
-  <si>
-    <t>Conhecimento</t>
-  </si>
-  <si>
-    <t>R$               34.420,70</t>
-  </si>
-  <si>
-    <t>Sessão de Julgamento TRT - Semipresencial</t>
-  </si>
-  <si>
-    <t>0011790-44.2024.5.15.0083</t>
-  </si>
-  <si>
-    <t>Kennedy Carvalho Lucas</t>
-  </si>
-  <si>
-    <t>02ª TURMA</t>
-  </si>
-  <si>
-    <t>Recursal TRT</t>
-  </si>
-  <si>
-    <t>R$             147.500,00</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/launch/jc/86986668664 ID da reunião: 869 8666 8664 Senha: 410044</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>0012495-75.2025.5.15.0093</t>
-  </si>
-  <si>
-    <t>Salitre Fertilizantes Ltda.</t>
-  </si>
-  <si>
-    <t>Eduardo Henrique Maia Carnauba</t>
-  </si>
-  <si>
-    <t>CAMPINAS</t>
-  </si>
-  <si>
-    <t>R$             596.014,50</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/81469918489?pwd=NmNHNVdhSERvZHorOXRIdmJCWU5MQT09 ID da reunião: 814 6991 8489 Senha: 059291</t>
-  </si>
-  <si>
-    <t>0010133-49.2026.5.15.0131</t>
-  </si>
-  <si>
-    <t>Alex Gomes De Sousa</t>
-  </si>
-  <si>
-    <t>12ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             179.903,44</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/86534999498?pwd=N3RZZXpkTE5laWxEREEvWjBVYVg0Zz0</t>
-  </si>
-  <si>
-    <t>0010841-17.2026.5.15.0126</t>
-  </si>
-  <si>
-    <t>Syngenta Proteção De Cultivos Ltda.</t>
-  </si>
-  <si>
-    <t>Claudinei Dos Santos</t>
-  </si>
-  <si>
-    <t>PAULÍNIA</t>
-  </si>
-  <si>
-    <t>R$               38.195,57</t>
-  </si>
-  <si>
-    <t>JPL</t>
-  </si>
-  <si>
-    <t>GVM</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/83059104477?pwd=h7VDkteaYgzZ4FIU9CoepcQo5ErUHA.1 ID da reunião: 830 5910 4477 Senha: 005974</t>
-  </si>
-  <si>
-    <t>0012011-90.2025.5.15.0083</t>
-  </si>
-  <si>
-    <t>Maria Fernanda Vila Nova Marson Schuller</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>R$             149.105,07</t>
-  </si>
-  <si>
-    <t>0011989-36.2024.5.15.0093</t>
-  </si>
-  <si>
-    <t>Gregory Ragosta Cassiano De Souza</t>
-  </si>
-  <si>
-    <t>05ª TURMA</t>
-  </si>
-  <si>
-    <t>Recursal</t>
-  </si>
-  <si>
-    <t>R$          1.066.473,00</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/88116222157?pwd=oFe1QBH0rStbUhO7ngHqYzIDE9abay.1</t>
-  </si>
-  <si>
-    <t>0010618-84.2026.5.15.0087</t>
-  </si>
-  <si>
-    <t>Rogerio Cordeiro</t>
-  </si>
-  <si>
-    <t>R$          1.150.491,32</t>
-  </si>
-  <si>
-    <t>JRM</t>
-  </si>
-  <si>
-    <t>https://trt15-jus-br.zoom.us/j/81792542599?pwd=dWt0TnU2UXVUYXdKTU1CU2gzUTVZQT09 ID da reunião: 817 9254 2599 Senha: 692443</t>
-  </si>
-  <si>
-    <t>0001673-47.2025.5.09.0011</t>
-  </si>
-  <si>
-    <t>Jose Aparecido Dos Santos Wermer</t>
-  </si>
-  <si>
-    <t>CURITIBA</t>
-  </si>
-  <si>
-    <t>11ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             303.594,35</t>
-  </si>
-  <si>
-    <t>RCF</t>
-  </si>
-  <si>
-    <t>1000994-20.2025.5.02.0433</t>
-  </si>
-  <si>
-    <t>Sidinei De Souza Oliveira</t>
-  </si>
-  <si>
-    <t>R$             400.000,00</t>
-  </si>
-  <si>
-    <t>0012474-76.2025.5.15.0133</t>
-  </si>
-  <si>
-    <t>Marcelo Luiz Teixeira</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DO RIO PRETO</t>
-  </si>
-  <si>
-    <t>Produção Antecipada de Prova</t>
-  </si>
-  <si>
-    <t>R$                    500,00</t>
+    <t>R$             281.252,53</t>
+  </si>
+  <si>
+    <t>Presencial | Advogada - Dra. Eliane Mendes, (15) 99949-8727</t>
   </si>
 </sst>
 </file>
@@ -1080,8 +1197,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49ED9DFC-A4C8-407F-936A-93E44AF2209F}">
-  <dimension ref="A1:R27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADEBBD58-7411-4639-9BF5-60AE082CEAAD}">
+  <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
@@ -1140,15 +1257,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>106140</v>
+        <v>93396</v>
       </c>
       <c r="B2" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C2" s="6">
-        <v>0.375</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -1192,19 +1309,19 @@
       <c r="Q2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>99850</v>
+        <v>106294</v>
       </c>
       <c r="B3" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C3" s="6">
-        <v>0.375</v>
+        <v>0.36180555555555555</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>33</v>
@@ -1222,13 +1339,13 @@
         <v>37</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>26</v>
@@ -1237,54 +1354,54 @@
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O3" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R3" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>106339</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q3" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>105023</v>
-      </c>
-      <c r="B4" s="5">
-        <v>46308</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0.375</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -1293,54 +1410,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
-        <v>105032</v>
+        <v>106292</v>
       </c>
       <c r="B5" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.37222222222222223</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1352,51 +1469,51 @@
         <v>59</v>
       </c>
       <c r="O5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>104126</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="Q5" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>105033</v>
-      </c>
-      <c r="B6" s="5">
-        <v>46308</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0.3923611111111111</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>62</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>55</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>63</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1405,54 +1522,54 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>32</v>
+        <v>69</v>
+      </c>
+      <c r="R6" s="8" t="s">
+        <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>104774</v>
+        <v>103238</v>
       </c>
       <c r="B7" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C7" s="6">
-        <v>0.39583333333333331</v>
+        <v>0.375</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>26</v>
@@ -1461,54 +1578,54 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>105223</v>
+        <v>103681</v>
       </c>
       <c r="B8" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C8" s="6">
-        <v>0.39583333333333331</v>
+        <v>0.375</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1517,54 +1634,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="R8" s="7" t="s">
-        <v>32</v>
+        <v>89</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>106263</v>
+        <v>104572</v>
       </c>
       <c r="B9" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C9" s="6">
-        <v>0.39583333333333331</v>
+        <v>0.38194444444444442</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>22</v>
+        <v>95</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1573,110 +1690,110 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="O9" s="7" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="Q9" s="7" t="s">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>32</v>
+        <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>99950</v>
+        <v>106004</v>
       </c>
       <c r="B10" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C10" s="6">
-        <v>0.41666666666666669</v>
+        <v>0.38958333333333334</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>37</v>
+        <v>103</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>41</v>
+        <v>106</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="R10" s="7" t="s">
-        <v>32</v>
+        <v>106</v>
+      </c>
+      <c r="R10" s="8" t="s">
+        <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>104771</v>
+        <v>105929</v>
       </c>
       <c r="B11" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C11" s="6">
-        <v>0.4201388888888889</v>
+        <v>0.40972222222222221</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>26</v>
@@ -1685,54 +1802,54 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="O11" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="Q11" s="7" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
-        <v>106063</v>
+        <v>105808</v>
       </c>
       <c r="B12" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C12" s="6">
-        <v>0.42708333333333331</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>43</v>
+        <v>108</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>103</v>
+        <v>47</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>38</v>
+        <v>118</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L12" s="7" t="s">
         <v>26</v>
@@ -1741,54 +1858,54 @@
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="R12" s="8" t="s">
-        <v>109</v>
+        <v>121</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>104667</v>
+        <v>103274</v>
       </c>
       <c r="B13" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C13" s="6">
-        <v>0.42708333333333331</v>
+        <v>0.4375</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>26</v>
@@ -1797,54 +1914,54 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>115</v>
+        <v>30</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="R13" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
+      </c>
+      <c r="R13" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>106100</v>
+        <v>93603</v>
       </c>
       <c r="B14" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C14" s="6">
-        <v>0.43055555555555558</v>
+        <v>0.44236111111111109</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>103</v>
+        <v>130</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>38</v>
+        <v>133</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>25</v>
+        <v>134</v>
       </c>
       <c r="L14" s="7" t="s">
         <v>26</v>
@@ -1853,54 +1970,54 @@
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>107</v>
+        <v>135</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>74</v>
+        <v>136</v>
       </c>
       <c r="P14" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>103106</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="Q14" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="R14" s="8" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4">
-        <v>105182</v>
-      </c>
-      <c r="B15" s="5">
-        <v>46308</v>
-      </c>
-      <c r="C15" s="6">
-        <v>0.47222222222222221</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>33</v>
-      </c>
       <c r="E15" s="7" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>22</v>
+        <v>142</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>26</v>
@@ -1909,54 +2026,54 @@
         <v>27</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>29</v>
+        <v>144</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>91</v>
+        <v>145</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>121</v>
+        <v>145</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>103551</v>
+        <v>100430</v>
       </c>
       <c r="B16" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C16" s="6">
-        <v>0.4861111111111111</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>33</v>
+        <v>146</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>26</v>
@@ -1965,54 +2082,54 @@
         <v>27</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="O16" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P16" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>104525</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="Q16" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="R16" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4">
-        <v>105174</v>
-      </c>
-      <c r="B17" s="5">
-        <v>46308</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0.5625</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>125</v>
-      </c>
       <c r="E17" s="7" t="s">
-        <v>126</v>
+        <v>153</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>127</v>
+        <v>47</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>128</v>
+        <v>154</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>105</v>
+        <v>49</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>106</v>
+        <v>23</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>129</v>
+        <v>40</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>26</v>
@@ -2021,54 +2138,54 @@
         <v>27</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>74</v>
+        <v>52</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="R17" s="8" t="s">
-        <v>109</v>
+        <v>106</v>
+      </c>
+      <c r="R17" s="7" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
-        <v>98816</v>
+        <v>104019</v>
       </c>
       <c r="B18" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C18" s="6">
-        <v>0.5625</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>131</v>
+        <v>71</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>55</v>
+        <v>157</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>57</v>
+        <v>159</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>134</v>
+        <v>39</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>135</v>
+        <v>40</v>
       </c>
       <c r="L18" s="7" t="s">
         <v>26</v>
@@ -2077,54 +2194,54 @@
         <v>27</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="R18" s="8" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
-        <v>103490</v>
+        <v>105287</v>
       </c>
       <c r="B19" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C19" s="6">
-        <v>0.58333333333333337</v>
+        <v>0.47986111111111113</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>138</v>
+        <v>91</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>140</v>
+        <v>93</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>142</v>
+        <v>95</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>113</v>
+        <v>164</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L19" s="7" t="s">
         <v>26</v>
@@ -2133,54 +2250,54 @@
         <v>27</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="R19" s="8" t="s">
-        <v>145</v>
+        <v>166</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
-        <v>103858</v>
+        <v>105649</v>
       </c>
       <c r="B20" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C20" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>142</v>
+        <v>169</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>148</v>
+        <v>76</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>25</v>
+        <v>113</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>26</v>
@@ -2189,54 +2306,54 @@
         <v>27</v>
       </c>
       <c r="N20" s="7" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="O20" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="Q20" s="7" t="s">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="R20" s="8" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
-        <v>105111</v>
+        <v>100814</v>
       </c>
       <c r="B21" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C21" s="6">
-        <v>0.59722222222222221</v>
+        <v>0.5444444444444444</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>138</v>
+        <v>81</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>154</v>
+        <v>64</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>72</v>
+        <v>175</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>83</v>
+        <v>176</v>
       </c>
       <c r="L21" s="7" t="s">
         <v>26</v>
@@ -2245,54 +2362,54 @@
         <v>27</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>40</v>
+        <v>178</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>156</v>
+        <v>54</v>
       </c>
       <c r="Q21" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="R21" s="8" t="s">
-        <v>158</v>
+        <v>54</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>179</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
-        <v>102063</v>
+        <v>100830</v>
       </c>
       <c r="B22" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C22" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>55</v>
+        <v>181</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>161</v>
+        <v>40</v>
       </c>
       <c r="L22" s="7" t="s">
         <v>26</v>
@@ -2301,54 +2418,54 @@
         <v>27</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>61</v>
+        <v>184</v>
       </c>
       <c r="Q22" s="7" t="s">
-        <v>86</v>
+        <v>185</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
-        <v>104088</v>
+        <v>105722</v>
       </c>
       <c r="B23" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C23" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.57986111111111116</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>131</v>
+        <v>33</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>111</v>
+        <v>187</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>142</v>
+        <v>189</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>23</v>
+        <v>190</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>165</v>
+        <v>39</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>166</v>
+        <v>40</v>
       </c>
       <c r="L23" s="7" t="s">
         <v>26</v>
@@ -2357,54 +2474,54 @@
         <v>27</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>51</v>
+        <v>192</v>
       </c>
       <c r="Q23" s="7" t="s">
-        <v>115</v>
+        <v>192</v>
       </c>
       <c r="R23" s="8" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
-        <v>104804</v>
+        <v>103736</v>
       </c>
       <c r="B24" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C24" s="6">
-        <v>0.61805555555555558</v>
+        <v>0.59027777777777779</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>152</v>
+        <v>195</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>170</v>
+        <v>196</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>154</v>
+        <v>197</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>23</v>
+        <v>198</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>89</v>
+        <v>199</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="L24" s="7" t="s">
         <v>26</v>
@@ -2413,54 +2530,54 @@
         <v>27</v>
       </c>
       <c r="N24" s="7" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="O24" s="7" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>156</v>
+        <v>201</v>
       </c>
       <c r="Q24" s="7" t="s">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="R24" s="8" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="96.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="259.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
-        <v>103582</v>
+        <v>105342</v>
       </c>
       <c r="B25" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C25" s="6">
-        <v>0.625</v>
+        <v>0.61805555555555558</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>45</v>
+        <v>205</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>176</v>
+        <v>207</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>161</v>
+        <v>113</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>26</v>
@@ -2469,54 +2586,54 @@
         <v>27</v>
       </c>
       <c r="N25" s="7" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="O25" s="7" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>179</v>
+        <v>78</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="R25" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="R25" s="8" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
-        <v>101364</v>
+        <v>101730</v>
       </c>
       <c r="B26" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C26" s="6">
-        <v>0.63888888888888884</v>
+        <v>0.625</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>20</v>
+        <v>211</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="L26" s="7" t="s">
         <v>26</v>
@@ -2525,92 +2642,151 @@
         <v>27</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>182</v>
+        <v>213</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>91</v>
+        <v>184</v>
       </c>
       <c r="Q26" s="7" t="s">
-        <v>31</v>
+        <v>184</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="173.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
-        <v>104114</v>
+        <v>105176</v>
       </c>
       <c r="B27" s="5">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C27" s="6">
-        <v>0.64583333333333337</v>
+        <v>0.63194444444444442</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>131</v>
+        <v>56</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>183</v>
+        <v>214</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>184</v>
+        <v>215</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>185</v>
+        <v>216</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>134</v>
+        <v>76</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>166</v>
+        <v>40</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>186</v>
+        <v>26</v>
       </c>
       <c r="M27" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N27" s="7" t="s">
-        <v>187</v>
+        <v>217</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>50</v>
+        <v>136</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>115</v>
+        <v>218</v>
       </c>
       <c r="Q27" s="7" t="s">
-        <v>115</v>
+        <v>218</v>
       </c>
       <c r="R27" s="8" t="s">
-        <v>137</v>
+        <v>219</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="84.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="4">
+        <v>102763</v>
+      </c>
+      <c r="B28" s="5">
+        <v>46309</v>
+      </c>
+      <c r="C28" s="6">
+        <v>0.65277777777777779</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N28" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="O28" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P28" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q28" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R28" s="7" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R4" r:id="rId1" xr:uid="{310473BB-B8CD-4DD8-8B8D-401BBE0BFB8D}"/>
-    <hyperlink ref="R7" r:id="rId2" xr:uid="{ADC369A2-DDBB-427A-8792-139A5490DAEB}"/>
-    <hyperlink ref="R12" r:id="rId3" xr:uid="{F5A0AD32-BCCB-4E63-97FF-CEEEA8E86AAB}"/>
-    <hyperlink ref="R14" r:id="rId4" xr:uid="{7C10BA1F-B68E-4AFB-8778-6CC1142B93A2}"/>
-    <hyperlink ref="R17" r:id="rId5" xr:uid="{96BB691E-FBB2-4A4D-8513-4B1CF0268199}"/>
-    <hyperlink ref="R18" r:id="rId6" xr:uid="{1B78F597-5AE0-4860-A993-4CEB4BF32486}"/>
-    <hyperlink ref="R19" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/81469918489?pwd=NmNHNVdhSERvZHorOXRIdmJCWU5MQT09%20ID%20da%20reunião:%20814%206991%208489%20Senha:%20059291" xr:uid="{54D7A758-1309-469C-B422-56A798998E2F}"/>
-    <hyperlink ref="R20" r:id="rId8" xr:uid="{A9451B6D-1FCD-4B0B-94BB-C1F1BD247588}"/>
-    <hyperlink ref="R21" r:id="rId9" display="https://trt15-jus-br.zoom.us/j/83059104477?pwd=h7VDkteaYgzZ4FIU9CoepcQo5ErUHA.1%20ID%20da%20reunião:%20830%205910%204477%20Senha:%20005974" xr:uid="{9A116859-DC0B-4508-A064-B9E8DFF3843D}"/>
-    <hyperlink ref="R23" r:id="rId10" xr:uid="{4CB3E34E-FC69-47E4-BCF5-7FE5E6492AD6}"/>
-    <hyperlink ref="R24" r:id="rId11" display="https://trt15-jus-br.zoom.us/j/81792542599?pwd=dWt0TnU2UXVUYXdKTU1CU2gzUTVZQT09%20ID%20da%20reunião:%20817%209254%202599%20Senha:%20692443" xr:uid="{59384DEE-FAC9-4D0C-B7ED-78FE9ABEF94D}"/>
-    <hyperlink ref="R27" r:id="rId12" xr:uid="{40C6B6EB-5908-4C50-8E3D-9AC500DFFA27}"/>
+    <hyperlink ref="R2" r:id="rId1" display="https://us02web.zoom.us/j/88415253122?pwd=QzlTNmxwdWpEeGVFZmdwM0lDUFJ4Zz09%20ID%20da%20reunião:%20884%201525%203122%20Senha%20de%20acesso:%20510562" xr:uid="{04C6DBE6-636E-40EE-A9EB-95E8083BE8AD}"/>
+    <hyperlink ref="R3" r:id="rId2" xr:uid="{2057B3DE-B348-4F28-B901-4051760C1203}"/>
+    <hyperlink ref="R5" r:id="rId3" xr:uid="{E6D4827D-77F9-4A6E-80A9-976EC081B772}"/>
+    <hyperlink ref="R6" r:id="rId4" xr:uid="{A0A7A5EC-227A-4E41-B500-1ED21846AA30}"/>
+    <hyperlink ref="R7" r:id="rId5" display="https://us02web.zoom.us/j/86212862282?pwd=N2N4b3NobCtXbUxsODdmSXFlMjVCQT09%20ID%20da%20reunião:%20862%201286%202282%20Senha:%20498067" xr:uid="{3F65D060-5C15-4917-A109-9585A087E950}"/>
+    <hyperlink ref="R8" r:id="rId6" xr:uid="{CE38DE43-E683-433B-9FF3-C44BE0670FF1}"/>
+    <hyperlink ref="R10" r:id="rId7" display="https://trt15-jus-br.zoom.us/j/85453506049?pwd=Q0lIZFc3eS9kaGNJQ3N0cEIxdnBnZz09%20ID%20da%20reunião:%20854%205350%206049%20Senha%20de%20acesso:%20364%20591" xr:uid="{0AF33F79-0A5A-4131-9FD9-111D9F8D07AB}"/>
+    <hyperlink ref="R13" r:id="rId8" display="https://trt5-jus-br.zoom.us/j/81333809109?pwd=47akSzaeNwYTr7VDOZiMN5qQCeHjkO.1%20ID%20da%20reunião:%20813%203380%209109%20Senha%20de%20acesso:%20470307" xr:uid="{C78255AE-E107-4464-B07C-8BE66868B575}"/>
+    <hyperlink ref="R18" r:id="rId9" xr:uid="{027F57A3-62AC-47FB-BA74-3D64A09D0B11}"/>
+    <hyperlink ref="R20" r:id="rId10" xr:uid="{A901F86D-862B-46F6-BE8E-DF824EC89DDB}"/>
+    <hyperlink ref="R23" r:id="rId11" display="https://trt23-jus-br.zoom.us/j/81753761549?pwd=NYkhI185ab9wC4FuLVDoNH2aVuBPb3.1%20ID%20da%20reunião:%20817%205376%201549%20Senha:%20@VTSinop1" xr:uid="{A13CD3B5-9027-462F-817B-1DC66274A514}"/>
+    <hyperlink ref="R24" r:id="rId12" display="https://trt9-jus-br.zoom.us/j/82898229693?pwd=WFk5UElWZGpDYjR0a1hTa2xwSHNjdz09%20ID%20reunião%20:%20828%209822%209693%20Senha%20de%20acesso:%20434474" xr:uid="{6B1AFD8E-17E0-4D3B-8646-70CE852D44F6}"/>
+    <hyperlink ref="R25" r:id="rId13" display="https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1%20ID%20da%20reunião:%20885%204267%202682%20Senha%20de%20acesso:%20050728" xr:uid="{8E3F3918-2EFE-4258-815D-3247602C5B70}"/>
+    <hyperlink ref="R27" r:id="rId14" xr:uid="{C0DAAC02-5281-481B-8717-21E720E9C40D}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Audiências: sync 2026-10-26 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5DB12E36-5FCC-40A3-9D1C-72A35A1AD21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{435E416E-2578-420A-B06D-D4446FC76848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29130" yWindow="4095" windowWidth="21600" windowHeight="11100" xr2:uid="{15D051F1-4BB8-4310-A08C-46B6246D8E3B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DCD763F2-081B-471F-BC06-16FA6600FB3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="152">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,22 +95,270 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Instrução - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011186-18.2026.5.15.0082</t>
+  </si>
+  <si>
+    <t>Moema Bioenergia S.A. - Moema</t>
+  </si>
+  <si>
+    <t>Adilson Maximiano Nogueira</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DO RIO PRETO</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$             112.227,97</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09 ID DA REUNIÃO: 817 5724 3738 SENHA: 954332</t>
+  </si>
+  <si>
     <t>Audiência Inicial -  Telepresencial</t>
   </si>
   <si>
-    <t>0000864-54.2026.5.23.0101</t>
+    <t>0011084-92.2026.5.03.0061</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Leandro Dos Santos</t>
+  </si>
+  <si>
+    <t>ITAJUBÁ</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>Ação de Consignação em Pagamento</t>
+  </si>
+  <si>
+    <t>R$                 3.262,69</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>TLI</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.itajuba</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0012242-06.2026.5.15.0044</t>
+  </si>
+  <si>
+    <t>Alessandre Lopes Da Cruz</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          2.819.517,97</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>0001518-55.2026.5.07.0014</t>
+  </si>
+  <si>
+    <t>Companhia Act De Participações E Companhia Aix De Participações.</t>
+  </si>
+  <si>
+    <t>Ana Angelica Nunes Nogueira Tavares</t>
+  </si>
+  <si>
+    <t>FORTALEZA</t>
+  </si>
+  <si>
+    <t>CE</t>
+  </si>
+  <si>
+    <t>14ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             100.200,00</t>
+  </si>
+  <si>
+    <t>Grupo C1</t>
+  </si>
+  <si>
+    <t>Correspondente - doc9</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Presencial | Advogado - Ikaro Handersson da Costa Farias </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF467886"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ikaro.handersson@gmail.com</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 85996385656 | Preposto - Ana Paula Barros Santos </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF467886"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>anapaulabarrossantos27@gmail.com</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (85)9982-60369</t>
+    </r>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0011691-29.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Pilkington Brasil Ltda.</t>
+  </si>
+  <si>
+    <t>Iraldenir De Oliveira Carneiro</t>
+  </si>
+  <si>
+    <t>CAÇAPAVA</t>
+  </si>
+  <si>
+    <t>R$               10.272,84</t>
+  </si>
+  <si>
+    <t>AAP</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>1001239-97.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>Elvis Filgueira De Almeida</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>R$             253.042,21</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>0011577-90.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Luis Jorge De Oliveira</t>
+  </si>
+  <si>
+    <t>R$                 3.658,27</t>
+  </si>
+  <si>
+    <t>0011552-77.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Ernani Rita De Oliveira</t>
+  </si>
+  <si>
+    <t>R$               56.941,59</t>
+  </si>
+  <si>
+    <t>0011549-25.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Marlene Santos Marcolino De Oliveira</t>
+  </si>
+  <si>
+    <t>R$               32.125,08</t>
+  </si>
+  <si>
+    <t>0010703-78.2026.5.03.0063</t>
   </si>
   <si>
     <t>Syngenta Seeds Ltda.</t>
   </si>
   <si>
-    <t>Iranildo Ferreira Alves Junior</t>
-  </si>
-  <si>
-    <t>LUCAS DO RIO VERDE</t>
-  </si>
-  <si>
-    <t>MT</t>
+    <t>Robert Da Silva Vilela</t>
+  </si>
+  <si>
+    <t>ITUIUTABA</t>
   </si>
   <si>
     <t>01ª VARA DO TRABALHO</t>
@@ -119,203 +367,179 @@
     <t>1ª Instância</t>
   </si>
   <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$               71.937,00</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
-  </si>
-  <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>GVM</t>
-  </si>
-  <si>
-    <t>https://trt23-jus-br.zoom.us/my/vtlucas1?pwd=RGxVbkdtRVE2TkllOHpmcEZ2NFd5UT09</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>1001652-34.2026.5.02.0037</t>
-  </si>
-  <si>
-    <t>Maricy Ciaccio Sichero</t>
-  </si>
-  <si>
-    <t>Ana Marilia Cassiano de Lima</t>
+    <t>R$               78.650,00</t>
+  </si>
+  <si>
+    <t>JRM</t>
+  </si>
+  <si>
+    <t>0011570-98.2025.5.15.0119</t>
+  </si>
+  <si>
+    <t>Martony Sampaio Ribeiro</t>
+  </si>
+  <si>
+    <t>R$               45.250,29</t>
+  </si>
+  <si>
+    <t>1001942-19.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Ryan Furtado Nascimento</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             157.873,36</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>NRG</t>
+  </si>
+  <si>
+    <t>1001442-50.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Luiz Gustavo Da Silva Buchmeier</t>
+  </si>
+  <si>
+    <t>R$                 7.632,80</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>1001441-71.2026.5.02.0433</t>
+  </si>
+  <si>
+    <t>Adonias Soares Da Silva</t>
+  </si>
+  <si>
+    <t>R$               51.027,24</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>0001305-77.2026.5.09.0019</t>
+  </si>
+  <si>
+    <t>Smartfit Escola De Ginastica E Danca S.A. E Bioritmo Franqueadora Ltda.</t>
+  </si>
+  <si>
+    <t>Neusa Aparecida Longuini</t>
+  </si>
+  <si>
+    <t>LONDRINA</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>CEJUSC</t>
+  </si>
+  <si>
+    <t>Reclamação Pré-processual</t>
+  </si>
+  <si>
+    <t>R$          2.418.775,20</t>
+  </si>
+  <si>
+    <t>Grupo A3</t>
+  </si>
+  <si>
+    <t>PBS</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/9kq15 ID da reunião: 82281762201 Senha de acesso: bOs5jU2nP7</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>1001886-19.2026.5.02.0521</t>
+  </si>
+  <si>
+    <t>Mahle Thermal And Fluid Systems Brazil Ltda.</t>
+  </si>
+  <si>
+    <t>Pamela Santana Borges Da Silva</t>
+  </si>
+  <si>
+    <t>ARUJÁ</t>
+  </si>
+  <si>
+    <t>R$                 5.367,99</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/87224949005?pwd=JbmIgbUoMHoknaZ0IapCSsc9JsarNK.1 ID da reunião: 872 2494 9005 Senha de acesso: vtaruja01</t>
+  </si>
+  <si>
+    <t>1001426-12.2025.5.02.0054</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Flavia Dias De Oliveira Faria</t>
   </si>
   <si>
     <t>SÃO PAULO</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>37ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>R$               35.016,39</t>
-  </si>
-  <si>
-    <t>Grupo C1</t>
-  </si>
-  <si>
-    <t>NBG</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>Audiência de Instrução - Telepresencial</t>
-  </si>
-  <si>
-    <t>1000642-34.2026.5.02.0431</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Bruno Alves Da Silva</t>
-  </si>
-  <si>
-    <t>SÃO CAETANO DO SUL</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          1.620.000,00</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/83190569296?pwd=YjNuL2d1T1dwNzJ0RGFjR0kveEpmQT09 ID da reunião: 831 9056 9296 Senha de acesso: sala2scs</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>0000770-07.2026.5.23.0037</t>
-  </si>
-  <si>
-    <t>Inpasa Agroindustrial S/A.</t>
-  </si>
-  <si>
-    <t>Bruna Silva De Oliveira</t>
-  </si>
-  <si>
-    <t>SINOP</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$               70.111,57</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>RRU</t>
-  </si>
-  <si>
-    <t>BTF</t>
-  </si>
-  <si>
-    <t>https://trt23-jus-br.zoom.us/j/3430107870?pwd=ZXR4a3MyUndBcjk0bnBDZ1lINThaQT09 ID da reunião: 343 010 7870 Senha de acesso: S6^vWi</t>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>1000618-51.2026.5.02.0319</t>
-  </si>
-  <si>
-    <t>Mahle Thermal And Fluid Systems Brazil Ltda.</t>
-  </si>
-  <si>
-    <t>Zivanildo Bezerra Barbosa</t>
-  </si>
-  <si>
-    <t>GUARULHOS</t>
-  </si>
-  <si>
-    <t>09ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             371.655,98</t>
-  </si>
-  <si>
-    <t>Correspondente - Carlos Florian</t>
-  </si>
-  <si>
-    <t>TLI</t>
-  </si>
-  <si>
-    <t>Presencial | Advogada - Dra. Ana Caroline, (11) 96079-1682</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Presencial</t>
-  </si>
-  <si>
-    <t>1001125-52.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>Junior Duarte Da Silva De Lima</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>R$             247.196,70</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>1001761-88.2025.5.02.0035</t>
-  </si>
-  <si>
-    <t>Willian Marcelino</t>
-  </si>
-  <si>
-    <t>35ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             573.120,80</t>
-  </si>
-  <si>
-    <t>ANB</t>
-  </si>
-  <si>
-    <t>GSM</t>
+    <t>54ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          2.092.449,00</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>0001611-58.2025.5.09.0673</t>
+  </si>
+  <si>
+    <t>Syngenta Comercial Agrícola Ltda.</t>
+  </si>
+  <si>
+    <t>Helio Ricardo Bruneri</t>
+  </si>
+  <si>
+    <t>06ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             249.131,93</t>
+  </si>
+  <si>
+    <t>VRO</t>
+  </si>
+  <si>
+    <t>0011431-10.2025.5.15.0132</t>
+  </si>
+  <si>
+    <t>Marcos Douglas Dos Santos Goulart</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>R$             376.645,91</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Ricardo de Souza Gonçalves ricardosgoncalves@live.com (12)9810-41449</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -333,6 +557,12 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF467886"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -424,7 +654,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -449,7 +679,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -786,8 +1016,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA5C575-525D-41DB-88BC-DA2048DBE0C9}">
-  <dimension ref="A1:R8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BCD8069-E596-41FB-A0B1-C8286F6CD83C}">
+  <dimension ref="A1:R20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
@@ -846,15 +1076,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>106051</v>
+        <v>104994</v>
       </c>
       <c r="B2" s="5">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="C2" s="6">
-        <v>0.34375</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -902,42 +1132,42 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>106674</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.34027777777777779</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="5">
-        <v>46318</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0.38194444444444442</v>
-      </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="K3" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="L3" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>26</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>27</v>
@@ -952,45 +1182,45 @@
         <v>44</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="R3" s="7" t="s">
         <v>45</v>
       </c>
+      <c r="R3" s="8" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>104654</v>
+        <v>105784</v>
       </c>
       <c r="B4" s="5">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="C4" s="6">
-        <v>0.4236111111111111</v>
+        <v>0.375</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>49</v>
       </c>
       <c r="H4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>51</v>
-      </c>
       <c r="K4" s="7" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="L4" s="7" t="s">
         <v>26</v>
@@ -999,54 +1229,54 @@
         <v>27</v>
       </c>
       <c r="N4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="240.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>106718</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.38194444444444442</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="Q4" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="R4" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>105716</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46318</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.4375</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>61</v>
-      </c>
       <c r="K5" s="7" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="L5" s="7" t="s">
         <v>26</v>
@@ -1055,54 +1285,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="P5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="R5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="Q5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>103635</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="R5" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>104580</v>
-      </c>
-      <c r="B6" s="5">
-        <v>46318</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0.5</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>71</v>
-      </c>
       <c r="I6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J6" s="7" t="s">
-        <v>72</v>
-      </c>
       <c r="K6" s="7" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1111,54 +1341,54 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>105256</v>
+        <v>105430</v>
       </c>
       <c r="B7" s="5">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="C7" s="6">
-        <v>0.51388888888888884</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>26</v>
@@ -1167,54 +1397,54 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="R7" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>103434</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="O7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="P7" s="7" t="s">
+      <c r="F8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="Q7" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
-        <v>103266</v>
-      </c>
-      <c r="B8" s="5">
-        <v>46318</v>
-      </c>
-      <c r="C8" s="6">
-        <v>0.51388888888888884</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>85</v>
-      </c>
       <c r="H8" s="7" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="I8" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>86</v>
-      </c>
       <c r="K8" s="7" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>26</v>
@@ -1223,26 +1453,701 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R8" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>103432</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.40277777777777779</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R9" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>103428</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="F10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="O10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P10" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R10" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>105581</v>
+      </c>
+      <c r="B11" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>103430</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R12" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>106323</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.4375</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="P8" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="R8" s="7" t="s">
+      <c r="E13" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q13" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="R13" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>105627</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P14" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q14" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="R14" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>105638</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q15" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="R15" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4">
+        <v>106665</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="4">
+        <v>105977</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.59375</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N17" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" s="7" t="s">
         <v>45</v>
+      </c>
+      <c r="Q17" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>104374</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="4">
+        <v>103660</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="O19" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="P19" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="R19" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4">
+        <v>101865</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="O20" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R20" s="8" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" xr:uid="{E11FDC00-DB29-40EE-AC70-ACC67E5FBE3B}"/>
-    <hyperlink ref="R4" r:id="rId2" display="https://trt2-jus-br.zoom.us/j/83190569296?pwd=YjNuL2d1T1dwNzJ0RGFjR0kveEpmQT09%20ID%20da%20reunião:%20831%209056%209296%20Senha%20de%20acesso:%20sala2scs" xr:uid="{A918178C-3043-43F2-9310-6FE1A651DFBA}"/>
-    <hyperlink ref="R5" r:id="rId3" display="https://trt23-jus-br.zoom.us/j/3430107870?pwd=ZXR4a3MyUndBcjk0bnBDZ1lINThaQT09%20ID%20da%20reunião:%20343%20010%207870%20Senha%20de%20acesso:%20S6%5evWi" xr:uid="{EED5B41A-F611-40DB-9FC0-9038D3BA52AF}"/>
+    <hyperlink ref="R2" r:id="rId1" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{9339D929-3BF8-4217-9323-72D4549FEB39}"/>
+    <hyperlink ref="R3" r:id="rId2" xr:uid="{C38F8162-A764-4CC8-BD09-5868F4A72B0F}"/>
+    <hyperlink ref="R4" r:id="rId3" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{A36F819B-3E41-410D-B38E-809C0AB943D8}"/>
+    <hyperlink ref="R16" r:id="rId4" xr:uid="{457C9B3A-A868-4E99-93B9-E5C29FF409A2}"/>
+    <hyperlink ref="R17" r:id="rId5" display="https://trt2-jus-br.zoom.us/j/87224949005?pwd=JbmIgbUoMHoknaZ0IapCSsc9JsarNK.1%20ID%20da%20reunião:%20872%202494%209005%20Senha%20de%20acesso:%20vtaruja01" xr:uid="{6B461923-48A8-4084-B100-CEDB0FD06DB7}"/>
+    <hyperlink ref="R20" r:id="rId6" display="mailto:ricardosgoncalves@live.com" xr:uid="{CD3B731A-48AF-47AF-B7D0-49E5F513C740}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Audiências: sync 2026-10-27 — Pauta de Audiências.xlsx
</commit_message>
<xml_diff>
--- a/Pauta_de_Audiencias.xlsx
+++ b/Pauta_de_Audiencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blu\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{435E416E-2578-420A-B06D-D4446FC76848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{168A89B5-15A8-49B6-B2A7-65065387B9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DCD763F2-081B-471F-BC06-16FA6600FB3D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{983DC53A-B337-4DA1-A7D8-F3264ADA8430}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="209">
   <si>
     <t>Código P&amp;C</t>
   </si>
@@ -95,146 +95,578 @@
     <t>Link/Observações</t>
   </si>
   <si>
+    <t>Audiência Una - Presencial</t>
+  </si>
+  <si>
+    <t>1001556-44.2026.5.02.0061</t>
+  </si>
+  <si>
+    <t>L. Sant'Angelo Pinturas Ltda</t>
+  </si>
+  <si>
+    <t>Marcos Leonio Fernandes De Queiroz</t>
+  </si>
+  <si>
+    <t>SÃO PAULO</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>61ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Instrução</t>
+  </si>
+  <si>
+    <t>Reclamação Trabalhista</t>
+  </si>
+  <si>
+    <t>CENTRAL</t>
+  </si>
+  <si>
+    <t>R$               32.163,75</t>
+  </si>
+  <si>
+    <t>Grupo E2</t>
+  </si>
+  <si>
+    <t>CAL</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Telepresencial</t>
+  </si>
+  <si>
+    <t>0000782-61.2026.5.05.0121</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda.</t>
+  </si>
+  <si>
+    <t>Emerson Souza Dos Santos</t>
+  </si>
+  <si>
+    <t>CANDEIAS</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$               68.299,07</t>
+  </si>
+  <si>
+    <t>MBF</t>
+  </si>
+  <si>
+    <t>https://trt5-jus-br.zoom.us/my/sl1vtca</t>
+  </si>
+  <si>
+    <t>Audiência Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0012613-54.2024.5.15.0071</t>
+  </si>
+  <si>
+    <t>Mahle Metal Leve S.A.</t>
+  </si>
+  <si>
+    <t>Wanderson Cunha Coelho</t>
+  </si>
+  <si>
+    <t>MOGI GUAÇU</t>
+  </si>
+  <si>
+    <t>Central</t>
+  </si>
+  <si>
+    <t>R$               78.909,58</t>
+  </si>
+  <si>
+    <t>Grupo E1</t>
+  </si>
+  <si>
+    <t>Correspondente - Ana Carolina Teresani</t>
+  </si>
+  <si>
+    <t>PSI</t>
+  </si>
+  <si>
+    <t>0010035-84.2025.5.15.0071</t>
+  </si>
+  <si>
+    <t>Maurilio Guilherme Dippre Macedo</t>
+  </si>
+  <si>
+    <t>R$             230.000,00</t>
+  </si>
+  <si>
+    <t>1002252-70.2025.5.02.0205</t>
+  </si>
+  <si>
+    <t>Alpha1 Empreendimento Imobiliario Spe Ltda</t>
+  </si>
+  <si>
+    <t>Lucas Correia Grageiro</t>
+  </si>
+  <si>
+    <t>BARUERI</t>
+  </si>
+  <si>
+    <t>05ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Conhecimento</t>
+  </si>
+  <si>
+    <t>R$               68.920,44</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>0017181-79.2025.5.15.0071</t>
+  </si>
+  <si>
+    <t>Ricardo Cesar Da Silva</t>
+  </si>
+  <si>
+    <t>Inicial</t>
+  </si>
+  <si>
+    <t>R$             501.217,75</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/5326391733?pwd=Qjc4RFBXWjZNbVd1bG5wNldjR3dWZz09</t>
+  </si>
+  <si>
+    <t>1000502-64.2026.5.02.0054</t>
+  </si>
+  <si>
+    <t>Telefonica Brasil S.A.</t>
+  </si>
+  <si>
+    <t>Barbara Servigne De Oliveira</t>
+  </si>
+  <si>
+    <t>54ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          1.172.734,00</t>
+  </si>
+  <si>
+    <t>Grupo C1</t>
+  </si>
+  <si>
+    <t>TFR</t>
+  </si>
+  <si>
+    <t>0011014-18.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Salitre Fertilizantes Ltda</t>
+  </si>
+  <si>
+    <t>Christian Monteiro Miranda</t>
+  </si>
+  <si>
+    <t>PATROCÍNIO</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>R$             143.700,00</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.patrocinio</t>
+  </si>
+  <si>
+    <t>0011015-03.2026.5.03.0080</t>
+  </si>
+  <si>
+    <t>Yury Goncalves De Oliveira</t>
+  </si>
+  <si>
+    <t>R$               77.600,00</t>
+  </si>
+  <si>
+    <t>1001284-08.2026.5.02.0463</t>
+  </si>
+  <si>
+    <t>Companhia Brasileira De Cartuchos</t>
+  </si>
+  <si>
+    <t>Moises De Mattos Damazio</t>
+  </si>
+  <si>
+    <t>SÃO BERNARDO DO CAMPO</t>
+  </si>
+  <si>
+    <t>03ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             132.745,00</t>
+  </si>
+  <si>
+    <t>Grupo B3</t>
+  </si>
+  <si>
+    <t>LMI</t>
+  </si>
+  <si>
+    <t>0010799-97.2026.5.15.0083</t>
+  </si>
+  <si>
+    <t>Embraer S.A.</t>
+  </si>
+  <si>
+    <t>Carlos Alberto Moreira Dos Santos</t>
+  </si>
+  <si>
+    <t>SÃO JOSÉ DOS CAMPOS</t>
+  </si>
+  <si>
+    <t>R$             133.051,44</t>
+  </si>
+  <si>
+    <t>Grupo B2</t>
+  </si>
+  <si>
+    <t>VCR</t>
+  </si>
+  <si>
+    <t>1001154-14.2026.5.02.0432</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
+  </si>
+  <si>
+    <t>David Henrique Silva Fernandes</t>
+  </si>
+  <si>
+    <t>SANTO ANDRÉ</t>
+  </si>
+  <si>
+    <t>04ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$          1.194.597,35</t>
+  </si>
+  <si>
+    <t>Grupo B1</t>
+  </si>
+  <si>
+    <t>Correspondente - Hebert</t>
+  </si>
+  <si>
+    <t>BSO</t>
+  </si>
+  <si>
+    <t>0010673-85.2026.5.15.0038</t>
+  </si>
+  <si>
+    <t>Steelcorp Construction S.A</t>
+  </si>
+  <si>
+    <t>Leonardo Papait Camilo</t>
+  </si>
+  <si>
+    <t>BRAGANÇA PAULISTA</t>
+  </si>
+  <si>
+    <t>R$             173.436,46</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>Audiência Inicial -  Presencial</t>
+  </si>
+  <si>
+    <t>1001030-34.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Marcio Jose Da Silva</t>
+  </si>
+  <si>
+    <t>R$          1.090.836,29</t>
+  </si>
+  <si>
+    <t>GSM</t>
+  </si>
+  <si>
+    <t>Sessão de Julgamento TRT - Presencial</t>
+  </si>
+  <si>
+    <t>1002143-77.2025.5.02.0004</t>
+  </si>
+  <si>
+    <t>Spic Brasil Energia Participações S.A.</t>
+  </si>
+  <si>
+    <t>Zenilda De Sousa Pinto</t>
+  </si>
+  <si>
+    <t>04ª TURMA</t>
+  </si>
+  <si>
+    <t>Recursal</t>
+  </si>
+  <si>
+    <t>R$               76.523,98</t>
+  </si>
+  <si>
+    <t>Grupo C2</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>ECO</t>
+  </si>
+  <si>
+    <t>0001807-67.2026.5.09.0002</t>
+  </si>
+  <si>
+    <t>Ferrero Do Brasil Industria Doceira E Alimentar Ltda.</t>
+  </si>
+  <si>
+    <t>Andreia Maria Gogola Albuquerque</t>
+  </si>
+  <si>
+    <t>CURITIBA</t>
+  </si>
+  <si>
+    <t>PR</t>
+  </si>
+  <si>
+    <t>02ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>R$             280.446,50</t>
+  </si>
+  <si>
+    <t>ANB</t>
+  </si>
+  <si>
+    <t>https://url.trt9.jus.br/ddx84 ID da Reunião: 82978782974 Senha: vg5XZiFlA1a</t>
+  </si>
+  <si>
+    <t>Audiência Inicial - Telepresencial</t>
+  </si>
+  <si>
+    <t>0010522-20.2026.5.15.0071</t>
+  </si>
+  <si>
+    <t>Paulo Cesar Torres Lopes</t>
+  </si>
+  <si>
+    <t>R$          1.453.867,32</t>
+  </si>
+  <si>
+    <t>ID da reunião: 532 639 1733 Senha de acesso: 959215</t>
+  </si>
+  <si>
+    <t>0010832-56.2026.5.03.0072</t>
+  </si>
+  <si>
+    <t>Usina Fotovoltaica Arinos</t>
+  </si>
+  <si>
+    <t>Leonardo Rocha Braga</t>
+  </si>
+  <si>
+    <t>UNAÍ</t>
+  </si>
+  <si>
+    <t>R$          1.018.759,39</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt.unai</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Telepresencial</t>
+  </si>
+  <si>
+    <t>1001576-77.2026.5.02.0435</t>
+  </si>
+  <si>
+    <t>Bridgestone Do Brasil Industria E Comercio Ltda.</t>
+  </si>
+  <si>
+    <t>Sidinei De Souza Oliveira</t>
+  </si>
+  <si>
+    <t>CEJUSC ABC</t>
+  </si>
+  <si>
+    <t>Cumprimento de Sentença</t>
+  </si>
+  <si>
+    <t>R$               19.517,93</t>
+  </si>
+  <si>
+    <t>JPE</t>
+  </si>
+  <si>
+    <t>https://trt2-jus-br.zoom.us/j/81881873237?pwd=aEs5S29DM2srNHRuRGFVM2ZEYkVUZz09 ID da reunião: 818 8187 3237 Senha de acesso: 459217</t>
+  </si>
+  <si>
+    <t>1001869-59.2026.5.02.0431</t>
+  </si>
+  <si>
+    <t>Wagner Goncalves Rosario</t>
+  </si>
+  <si>
+    <t>R$          1.064.563,78</t>
+  </si>
+  <si>
+    <t>RFE</t>
+  </si>
+  <si>
+    <t>1000886-24.2026.5.02.0443</t>
+  </si>
+  <si>
+    <t>Syngenta Proteção De Cultivos Ltda.</t>
+  </si>
+  <si>
+    <t>Everton Antonio Candido Nunes</t>
+  </si>
+  <si>
+    <t>SANTOS</t>
+  </si>
+  <si>
+    <t>1ª Instância</t>
+  </si>
+  <si>
+    <t>R$             123.100,00</t>
+  </si>
+  <si>
+    <t>Correspondente - Carlos Florian</t>
+  </si>
+  <si>
+    <t>GVM</t>
+  </si>
+  <si>
+    <t>Presencial | Advogado - Dr. Gustavo Barker, (13) 98181-1004 | Preposto - Milena Antunes dos Santos, CPF 306.966.018-50, RG 349608027, (13) 99709-1342</t>
+  </si>
+  <si>
+    <t>Audiência Una - Telepresencial</t>
+  </si>
+  <si>
+    <t>0011305-74.2026.5.03.0029</t>
+  </si>
+  <si>
+    <t>Sistenge Construcoes E Comercio Ltda</t>
+  </si>
+  <si>
+    <t>Jeronimo De Barros</t>
+  </si>
+  <si>
+    <t>CONTAGEM</t>
+  </si>
+  <si>
+    <t>01ª VARA DO TRABALHO</t>
+  </si>
+  <si>
+    <t>Acordo</t>
+  </si>
+  <si>
+    <t>R$               43.815,14</t>
+  </si>
+  <si>
+    <t>RYL</t>
+  </si>
+  <si>
+    <t>https://trt3-jus-br.zoom.us/my/vt1.contagem</t>
+  </si>
+  <si>
     <t>Audiência Instrução - Telepresencial</t>
   </si>
   <si>
-    <t>0011186-18.2026.5.15.0082</t>
+    <t>0010866-65.2026.5.15.0082</t>
   </si>
   <si>
     <t>Moema Bioenergia S.A. - Moema</t>
   </si>
   <si>
-    <t>Adilson Maximiano Nogueira</t>
+    <t>Antonio Osorio Sontin Ferreira</t>
   </si>
   <si>
     <t>SÃO JOSÉ DO RIO PRETO</t>
   </si>
   <si>
-    <t>SP</t>
-  </si>
-  <si>
-    <t>03ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Instrução</t>
-  </si>
-  <si>
-    <t>Reclamação Trabalhista</t>
-  </si>
-  <si>
-    <t>CENTRAL</t>
-  </si>
-  <si>
-    <t>R$             112.227,97</t>
-  </si>
-  <si>
-    <t>Grupo E2</t>
-  </si>
-  <si>
-    <t>MBF</t>
-  </si>
-  <si>
-    <t>RYL</t>
-  </si>
-  <si>
-    <t>https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09 ID DA REUNIÃO: 817 5724 3738 SENHA: 954332</t>
-  </si>
-  <si>
-    <t>Audiência Inicial -  Telepresencial</t>
-  </si>
-  <si>
-    <t>0011084-92.2026.5.03.0061</t>
-  </si>
-  <si>
-    <t>Mahle Metal Leve S.A.</t>
-  </si>
-  <si>
-    <t>Leandro Dos Santos</t>
-  </si>
-  <si>
-    <t>ITAJUBÁ</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>Inicial</t>
-  </si>
-  <si>
-    <t>Ação de Consignação em Pagamento</t>
-  </si>
-  <si>
-    <t>R$                 3.262,69</t>
-  </si>
-  <si>
-    <t>Grupo E1</t>
+    <t>R$             254.000,00</t>
+  </si>
+  <si>
+    <t>https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1 ID da reunião: 885 4267 2682 Senha de acesso: 50728</t>
+  </si>
+  <si>
+    <t>Audiência de Conciliação - Semipresencial</t>
+  </si>
+  <si>
+    <t>0011309-25.2019.5.15.0126</t>
+  </si>
+  <si>
+    <t>Wagner De Jesus Sena</t>
+  </si>
+  <si>
+    <t>PAULÍNIA</t>
+  </si>
+  <si>
+    <t>CEJUSC CAMPINAS</t>
+  </si>
+  <si>
+    <t>Execução</t>
+  </si>
+  <si>
+    <t>R$                 9.489,28</t>
   </si>
   <si>
     <t>TLI</t>
   </si>
   <si>
-    <t>PSI</t>
-  </si>
-  <si>
-    <t>https://trt3-jus-br.zoom.us/my/vt.itajuba</t>
-  </si>
-  <si>
-    <t>Audiência Inicial - Telepresencial</t>
-  </si>
-  <si>
-    <t>0012242-06.2026.5.15.0044</t>
-  </si>
-  <si>
-    <t>Alessandre Lopes Da Cruz</t>
-  </si>
-  <si>
-    <t>02ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          2.819.517,97</t>
-  </si>
-  <si>
-    <t>ARC</t>
-  </si>
-  <si>
-    <t>Audiência Una - Presencial</t>
-  </si>
-  <si>
-    <t>0001518-55.2026.5.07.0014</t>
-  </si>
-  <si>
-    <t>Companhia Act De Participações E Companhia Aix De Participações.</t>
-  </si>
-  <si>
-    <t>Ana Angelica Nunes Nogueira Tavares</t>
-  </si>
-  <si>
-    <t>FORTALEZA</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>14ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             100.200,00</t>
-  </si>
-  <si>
-    <t>Grupo C1</t>
+    <t>https://trt15-jus-br.zoom.us/j/88582969985?pwd=KDz0bWgxYzvepXfQC3ZYK8t4t1RyOY.1 ID: 885 8296 9985 Senha: 3</t>
+  </si>
+  <si>
+    <t>Audiência de Instrução - Presencial</t>
+  </si>
+  <si>
+    <t>0010821-92.2025.5.15.0083</t>
+  </si>
+  <si>
+    <t>Julio Cesar De Souza</t>
+  </si>
+  <si>
+    <t>R$             100.000,00</t>
+  </si>
+  <si>
+    <t>0010417-72.2026.5.15.0029</t>
+  </si>
+  <si>
+    <t>Viterra Bioenergia S.A.</t>
+  </si>
+  <si>
+    <t>Daniel Antonio</t>
+  </si>
+  <si>
+    <t>JABOTICABAL</t>
+  </si>
+  <si>
+    <t>R$          1.318.000,00</t>
   </si>
   <si>
     <t>Correspondente - doc9</t>
   </si>
   <si>
-    <t>VSI</t>
-  </si>
-  <si>
     <r>
-      <t xml:space="preserve">Presencial | Advogado - Ikaro Handersson da Costa Farias </t>
+      <t xml:space="preserve">Presencial | Advogado - David Barbosa Botelho </t>
     </r>
     <r>
       <rPr>
@@ -243,7 +675,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>ikaro.handersson@gmail.com</t>
+      <t>davidbarbosa572@gmail.com</t>
     </r>
     <r>
       <rPr>
@@ -252,7 +684,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> 85996385656 | Preposto - Ana Paula Barros Santos </t>
+      <t xml:space="preserve"> (16)9999-23722 | Preposto - Nayane Gambi Cezano Barbosa </t>
     </r>
     <r>
       <rPr>
@@ -261,7 +693,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>anapaulabarrossantos27@gmail.com</t>
+      <t>dra.nayanegambi@gmail.com</t>
     </r>
     <r>
       <rPr>
@@ -270,269 +702,8 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> (85)9982-60369</t>
+      <t xml:space="preserve"> (16)99164-5306</t>
     </r>
-  </si>
-  <si>
-    <t>Audiência Instrução - Presencial</t>
-  </si>
-  <si>
-    <t>0011691-29.2025.5.15.0119</t>
-  </si>
-  <si>
-    <t>Pilkington Brasil Ltda.</t>
-  </si>
-  <si>
-    <t>Iraldenir De Oliveira Carneiro</t>
-  </si>
-  <si>
-    <t>CAÇAPAVA</t>
-  </si>
-  <si>
-    <t>R$               10.272,84</t>
-  </si>
-  <si>
-    <t>AAP</t>
-  </si>
-  <si>
-    <t>Presencial</t>
-  </si>
-  <si>
-    <t>1001239-97.2026.5.02.0432</t>
-  </si>
-  <si>
-    <t>Bridgestone Do Brasil Indústria E Comércio Ltda.</t>
-  </si>
-  <si>
-    <t>Elvis Filgueira De Almeida</t>
-  </si>
-  <si>
-    <t>SANTO ANDRÉ</t>
-  </si>
-  <si>
-    <t>R$             253.042,21</t>
-  </si>
-  <si>
-    <t>Grupo B1</t>
-  </si>
-  <si>
-    <t>GSM</t>
-  </si>
-  <si>
-    <t>BSO</t>
-  </si>
-  <si>
-    <t>0011577-90.2025.5.15.0119</t>
-  </si>
-  <si>
-    <t>Luis Jorge De Oliveira</t>
-  </si>
-  <si>
-    <t>R$                 3.658,27</t>
-  </si>
-  <si>
-    <t>0011552-77.2025.5.15.0119</t>
-  </si>
-  <si>
-    <t>Ernani Rita De Oliveira</t>
-  </si>
-  <si>
-    <t>R$               56.941,59</t>
-  </si>
-  <si>
-    <t>0011549-25.2025.5.15.0119</t>
-  </si>
-  <si>
-    <t>Marlene Santos Marcolino De Oliveira</t>
-  </si>
-  <si>
-    <t>R$               32.125,08</t>
-  </si>
-  <si>
-    <t>0010703-78.2026.5.03.0063</t>
-  </si>
-  <si>
-    <t>Syngenta Seeds Ltda.</t>
-  </si>
-  <si>
-    <t>Robert Da Silva Vilela</t>
-  </si>
-  <si>
-    <t>ITUIUTABA</t>
-  </si>
-  <si>
-    <t>01ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>1ª Instância</t>
-  </si>
-  <si>
-    <t>R$               78.650,00</t>
-  </si>
-  <si>
-    <t>JRM</t>
-  </si>
-  <si>
-    <t>0011570-98.2025.5.15.0119</t>
-  </si>
-  <si>
-    <t>Martony Sampaio Ribeiro</t>
-  </si>
-  <si>
-    <t>R$               45.250,29</t>
-  </si>
-  <si>
-    <t>1001942-19.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>Ryan Furtado Nascimento</t>
-  </si>
-  <si>
-    <t>05ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             157.873,36</t>
-  </si>
-  <si>
-    <t>Correspondente - Hebert</t>
-  </si>
-  <si>
-    <t>NRG</t>
-  </si>
-  <si>
-    <t>1001442-50.2026.5.02.0435</t>
-  </si>
-  <si>
-    <t>Luiz Gustavo Da Silva Buchmeier</t>
-  </si>
-  <si>
-    <t>R$                 7.632,80</t>
-  </si>
-  <si>
-    <t>RFE</t>
-  </si>
-  <si>
-    <t>1001441-71.2026.5.02.0433</t>
-  </si>
-  <si>
-    <t>Adonias Soares Da Silva</t>
-  </si>
-  <si>
-    <t>R$               51.027,24</t>
-  </si>
-  <si>
-    <t>LMI</t>
-  </si>
-  <si>
-    <t>Audiência de Conciliação - Telepresencial</t>
-  </si>
-  <si>
-    <t>0001305-77.2026.5.09.0019</t>
-  </si>
-  <si>
-    <t>Smartfit Escola De Ginastica E Danca S.A. E Bioritmo Franqueadora Ltda.</t>
-  </si>
-  <si>
-    <t>Neusa Aparecida Longuini</t>
-  </si>
-  <si>
-    <t>LONDRINA</t>
-  </si>
-  <si>
-    <t>PR</t>
-  </si>
-  <si>
-    <t>CEJUSC</t>
-  </si>
-  <si>
-    <t>Reclamação Pré-processual</t>
-  </si>
-  <si>
-    <t>R$          2.418.775,20</t>
-  </si>
-  <si>
-    <t>Grupo A3</t>
-  </si>
-  <si>
-    <t>PBS</t>
-  </si>
-  <si>
-    <t>https://url.trt9.jus.br/9kq15 ID da reunião: 82281762201 Senha de acesso: bOs5jU2nP7</t>
-  </si>
-  <si>
-    <t>Audiência Una - Telepresencial</t>
-  </si>
-  <si>
-    <t>1001886-19.2026.5.02.0521</t>
-  </si>
-  <si>
-    <t>Mahle Thermal And Fluid Systems Brazil Ltda.</t>
-  </si>
-  <si>
-    <t>Pamela Santana Borges Da Silva</t>
-  </si>
-  <si>
-    <t>ARUJÁ</t>
-  </si>
-  <si>
-    <t>R$                 5.367,99</t>
-  </si>
-  <si>
-    <t>https://trt2-jus-br.zoom.us/j/87224949005?pwd=JbmIgbUoMHoknaZ0IapCSsc9JsarNK.1 ID da reunião: 872 2494 9005 Senha de acesso: vtaruja01</t>
-  </si>
-  <si>
-    <t>1001426-12.2025.5.02.0054</t>
-  </si>
-  <si>
-    <t>Telefonica Brasil S.A.</t>
-  </si>
-  <si>
-    <t>Flavia Dias De Oliveira Faria</t>
-  </si>
-  <si>
-    <t>SÃO PAULO</t>
-  </si>
-  <si>
-    <t>54ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$          2.092.449,00</t>
-  </si>
-  <si>
-    <t>TFR</t>
-  </si>
-  <si>
-    <t>0001611-58.2025.5.09.0673</t>
-  </si>
-  <si>
-    <t>Syngenta Comercial Agrícola Ltda.</t>
-  </si>
-  <si>
-    <t>Helio Ricardo Bruneri</t>
-  </si>
-  <si>
-    <t>06ª VARA DO TRABALHO</t>
-  </si>
-  <si>
-    <t>R$             249.131,93</t>
-  </si>
-  <si>
-    <t>VRO</t>
-  </si>
-  <si>
-    <t>0011431-10.2025.5.15.0132</t>
-  </si>
-  <si>
-    <t>Marcos Douglas Dos Santos Goulart</t>
-  </si>
-  <si>
-    <t>SÃO JOSÉ DOS CAMPOS</t>
-  </si>
-  <si>
-    <t>R$             376.645,91</t>
-  </si>
-  <si>
-    <t>Presencial | Advogado - Ricardo de Souza Gonçalves ricardosgoncalves@live.com (12)9810-41449</t>
   </si>
 </sst>
 </file>
@@ -1016,8 +1187,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BCD8069-E596-41FB-A0B1-C8286F6CD83C}">
-  <dimension ref="A1:R20"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C7AF8A9-DF41-4891-9826-70D604F0E7F0}">
+  <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:18" ht="60" x14ac:dyDescent="0.3">
@@ -1076,15 +1247,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
-        <v>104994</v>
+        <v>106065</v>
       </c>
       <c r="B2" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C2" s="6">
-        <v>0.33333333333333331</v>
+        <v>0.34722222222222221</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>18</v>
@@ -1126,98 +1297,98 @@
         <v>30</v>
       </c>
       <c r="Q2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="R2" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
-        <v>106674</v>
+        <v>105789</v>
       </c>
       <c r="B3" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C3" s="6">
-        <v>0.34027777777777779</v>
+        <v>0.37152777777777779</v>
       </c>
       <c r="D3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="7" t="s">
-        <v>39</v>
-      </c>
       <c r="K3" s="7" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
-        <v>105784</v>
+        <v>99614</v>
       </c>
       <c r="B4" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C4" s="6">
         <v>0.375</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>25</v>
@@ -1226,54 +1397,54 @@
         <v>26</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="N4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="O4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="7" t="s">
+      <c r="R4" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>100140</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="240.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>106718</v>
-      </c>
-      <c r="B5" s="5">
-        <v>46321</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.38194444444444442</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>56</v>
-      </c>
       <c r="H5" s="7" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>25</v>
@@ -1285,54 +1456,54 @@
         <v>27</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="Q5" s="7" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>64</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
-        <v>103635</v>
+        <v>105923</v>
       </c>
       <c r="B6" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C6" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>26</v>
@@ -1341,54 +1512,54 @@
         <v>27</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="O6" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="Q6" s="7" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
-        <v>105430</v>
+        <v>103541</v>
       </c>
       <c r="B7" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C7" s="6">
-        <v>0.3888888888888889</v>
+        <v>0.41319444444444442</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>74</v>
+        <v>44</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>26</v>
@@ -1397,51 +1568,51 @@
         <v>27</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="Q7" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="R7" s="7" t="s">
-        <v>72</v>
+        <v>51</v>
+      </c>
+      <c r="R7" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
-        <v>103434</v>
+        <v>104752</v>
       </c>
       <c r="B8" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C8" s="6">
-        <v>0.39583333333333331</v>
+        <v>0.4236111111111111</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>25</v>
@@ -1453,54 +1624,54 @@
         <v>27</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="Q8" s="7" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
-        <v>103432</v>
+        <v>105968</v>
       </c>
       <c r="B9" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C9" s="6">
-        <v>0.40277777777777779</v>
+        <v>0.4236111111111111</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="L9" s="7" t="s">
         <v>26</v>
@@ -1509,54 +1680,54 @@
         <v>27</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="O9" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="Q9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="R9" s="7" t="s">
-        <v>72</v>
+      <c r="R9" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
-        <v>103428</v>
+        <v>105967</v>
       </c>
       <c r="B10" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C10" s="6">
-        <v>0.41319444444444442</v>
+        <v>0.42708333333333331</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>26</v>
@@ -1565,54 +1736,54 @@
         <v>27</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="O10" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="Q10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="R10" s="7" t="s">
-        <v>72</v>
+      <c r="R10" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
-        <v>105581</v>
+        <v>105741</v>
       </c>
       <c r="B11" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C11" s="6">
-        <v>0.42708333333333331</v>
+        <v>0.43055555555555558</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>26</v>
@@ -1621,51 +1792,51 @@
         <v>27</v>
       </c>
       <c r="N11" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O11" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="P11" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q11" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>104798</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.4375</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="H12" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="O11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="P11" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q11" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4">
-        <v>103430</v>
-      </c>
-      <c r="B12" s="5">
-        <v>46321</v>
-      </c>
-      <c r="C12" s="6">
-        <v>0.43055555555555558</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>69</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>25</v>
@@ -1677,51 +1848,51 @@
         <v>27</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O12" s="7" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
-        <v>106323</v>
+        <v>105292</v>
       </c>
       <c r="B13" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C13" s="6">
-        <v>0.4375</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E13" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>74</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>102</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>25</v>
@@ -1733,107 +1904,107 @@
         <v>27</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O13" s="7" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="Q13" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
-        <v>105627</v>
+        <v>105221</v>
       </c>
       <c r="B14" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C14" s="6">
-        <v>0.44444444444444442</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>103</v>
+        <v>38</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O14" s="7" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="Q14" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
-        <v>105638</v>
+        <v>105139</v>
       </c>
       <c r="B15" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C15" s="6">
-        <v>0.45833333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>53</v>
+        <v>115</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>74</v>
+        <v>101</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>25</v>
@@ -1845,110 +2016,110 @@
         <v>27</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="O15" s="7" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="Q15" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="159" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
-        <v>106665</v>
+        <v>103634</v>
       </c>
       <c r="B16" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C16" s="6">
         <v>0.54166666666666663</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>119</v>
+        <v>22</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>120</v>
+        <v>23</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="O16" s="7" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="Q16" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="R16" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="144.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
-        <v>105977</v>
+        <v>106702</v>
       </c>
       <c r="B17" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C17" s="6">
-        <v>0.59375</v>
+        <v>0.54305555555555551</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>127</v>
+        <v>32</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>23</v>
+        <v>134</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>39</v>
+        <v>135</v>
       </c>
       <c r="K17" s="7" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="L17" s="7" t="s">
         <v>26</v>
@@ -1957,54 +2128,54 @@
         <v>27</v>
       </c>
       <c r="N17" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="O17" s="7" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>45</v>
+        <v>137</v>
       </c>
       <c r="Q17" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="R17" s="8" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="4">
+        <v>104515</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="R17" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4">
-        <v>104374</v>
-      </c>
-      <c r="B18" s="5">
-        <v>46321</v>
-      </c>
-      <c r="C18" s="6">
-        <v>0.59722222222222221</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>135</v>
-      </c>
       <c r="G18" s="7" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>137</v>
+        <v>46</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>138</v>
+        <v>38</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="L18" s="7" t="s">
         <v>26</v>
@@ -2013,54 +2184,54 @@
         <v>27</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
       <c r="Q18" s="7" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>72</v>
+        <v>143</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
-        <v>103660</v>
+        <v>106156</v>
       </c>
       <c r="B19" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C19" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.5625</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>119</v>
+        <v>147</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>120</v>
+        <v>79</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>144</v>
+        <v>38</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="L19" s="7" t="s">
         <v>26</v>
@@ -2069,85 +2240,481 @@
         <v>27</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="Q19" s="7" t="s">
-        <v>146</v>
-      </c>
-      <c r="R19" s="7" t="s">
-        <v>72</v>
+        <v>129</v>
+      </c>
+      <c r="R19" s="8" t="s">
+        <v>149</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="245.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
-        <v>101865</v>
+        <v>105940</v>
       </c>
       <c r="B20" s="5">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C20" s="6">
-        <v>0.60416666666666663</v>
+        <v>0.5708333333333333</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>53</v>
+        <v>150</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>149</v>
+        <v>103</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>23</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>25</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>26</v>
+        <v>155</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>27</v>
       </c>
       <c r="N20" s="7" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="O20" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="P20" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="Q20" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="R20" s="8" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4">
+        <v>106206</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C21" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="K21" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L21" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="O21" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="P21" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q21" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="R21" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="192.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4">
+        <v>105491</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C22" s="6">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="O22" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="P22" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q22" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="R22" s="7" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4">
+        <v>105540</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.59791666666666665</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K23" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="O23" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="P20" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q20" s="7" t="s">
+      <c r="P23" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q23" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="R23" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="259.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4">
+        <v>104926</v>
+      </c>
+      <c r="B24" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C24" s="6">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L24" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N24" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="O24" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q24" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="R20" s="8" t="s">
-        <v>151</v>
+      <c r="R24" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="202.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4">
+        <v>74935</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C25" s="6">
+        <v>0.62013888888888891</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="L25" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="N25" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="P25" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q25" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="R25" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>106219</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0.625</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L26" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N26" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="P26" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q26" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="R26" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="240.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="4">
+        <v>104781</v>
+      </c>
+      <c r="B27" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0.65277777777777779</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L27" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N27" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="O27" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P27" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="R27" s="7" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R2" r:id="rId1" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{9339D929-3BF8-4217-9323-72D4549FEB39}"/>
-    <hyperlink ref="R3" r:id="rId2" xr:uid="{C38F8162-A764-4CC8-BD09-5868F4A72B0F}"/>
-    <hyperlink ref="R4" r:id="rId3" display="https://us02web.zoom.us/j/81757243738?pwd=UXAvdEpveHlrNU05M2ZsZnRrYy9Vdz09%20ID%20DA%20REUNIÃO:%20817%205724%203738%20SENHA:%20954332" xr:uid="{A36F819B-3E41-410D-B38E-809C0AB943D8}"/>
-    <hyperlink ref="R16" r:id="rId4" xr:uid="{457C9B3A-A868-4E99-93B9-E5C29FF409A2}"/>
-    <hyperlink ref="R17" r:id="rId5" display="https://trt2-jus-br.zoom.us/j/87224949005?pwd=JbmIgbUoMHoknaZ0IapCSsc9JsarNK.1%20ID%20da%20reunião:%20872%202494%209005%20Senha%20de%20acesso:%20vtaruja01" xr:uid="{6B461923-48A8-4084-B100-CEDB0FD06DB7}"/>
-    <hyperlink ref="R20" r:id="rId6" display="mailto:ricardosgoncalves@live.com" xr:uid="{CD3B731A-48AF-47AF-B7D0-49E5F513C740}"/>
+    <hyperlink ref="R3" r:id="rId1" xr:uid="{E70C753C-B4AB-4DA2-8874-4D6BE15AEE9C}"/>
+    <hyperlink ref="R7" r:id="rId2" xr:uid="{8CD7349B-B768-4F32-97AD-E4C6B17FDF28}"/>
+    <hyperlink ref="R9" r:id="rId3" xr:uid="{1FEAC607-4DCB-4486-8328-9D7EE3CCD37E}"/>
+    <hyperlink ref="R10" r:id="rId4" xr:uid="{1164ACF0-76E2-4389-B572-4DED5239179C}"/>
+    <hyperlink ref="R17" r:id="rId5" xr:uid="{29BE04FB-4A65-49E6-A5EC-7CBD5FAA6837}"/>
+    <hyperlink ref="R19" r:id="rId6" xr:uid="{E56E5952-F400-4F88-A83D-F445B892AC2D}"/>
+    <hyperlink ref="R20" r:id="rId7" display="https://trt2-jus-br.zoom.us/j/81881873237?pwd=aEs5S29DM2srNHRuRGFVM2ZEYkVUZz09%20ID%20da%20reunião:%20818%208187%203237%20Senha%20de%20acesso:%20459217" xr:uid="{B2D22885-963B-4781-8C82-82555603F2AB}"/>
+    <hyperlink ref="R23" r:id="rId8" xr:uid="{11F48EB9-0F83-4108-87F4-CD040B1657FC}"/>
+    <hyperlink ref="R24" r:id="rId9" display="https://trt15-jus-br.zoom.us/j/88542672682?pwd=7pQ4QRhZmRG9RAQAWKowymbwNawa7t.1%20ID%20da%20reunião:%20885%204267%202682%20Senha%20de%20acesso:%2050728" xr:uid="{FEFA1AE1-4656-432D-92AC-8A5CABB385F7}"/>
+    <hyperlink ref="R25" r:id="rId10" display="https://trt15-jus-br.zoom.us/j/88582969985?pwd=KDz0bWgxYzvepXfQC3ZYK8t4t1RyOY.1%20ID:%20885%208296%209985%20Senha:%203" xr:uid="{65EE2F3D-CFA0-436B-B350-CD4ACCF5342D}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>